<commit_message>
Model in-house media: architecture D, broker time, and shooting capacity
Adds the case where the broker shoots listing media himself: $65 editing plus
flyers and sign/lockbox is $210 cash per listing, versus $720 outsourced. Also
adds the two costs that case hides — the broker's hours per listing valued at an
opportunity rate, and a monthly shooting capacity above which overflow is
outsourced at full price. A switch lets you see the flattering version where
your own labor is free.

Findings: at $399 per transaction the monthly fee, not the media, is what
decides viability. $29/month needs 36 agents to break even, $99/month needs 12.
Listing contribution is still -$42 at $99 once the broker's time is counted;
a $149 per-listing media fee charged to the agent flips it to +$108 and pulls
break-even to 9 agents.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -1229,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1472,72 +1472,102 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Monthly fee — D (in-house media)</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>99</v>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>The per-seat tech stack costs about $83 a month. A $20 fee cannot cover it; this one can.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Transaction fee — D</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>399</v>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Your number, kept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Blended economics at the selected architecture and scenario</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="20" t="n"/>
-      <c r="I18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Blended monthly fee per agent</t>
-        </is>
-      </c>
-      <c r="B19" s="21">
-        <f>IF($B$3="B. Tiered",B6*Scenarios!$E$14+C6*Scenarios!$E$15+D6*Scenarios!$E$16,B13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Blended transaction fee</t>
-        </is>
-      </c>
-      <c r="B20" s="21">
-        <f>IF($B$3="B. Tiered",B7*Scenarios!$E$14+C7*Scenarios!$E$15+D7*Scenarios!$E$16,B14)</f>
-        <v/>
-      </c>
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="20" t="n"/>
+      <c r="G20" s="20" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Blended media credit per listing</t>
+          <t>Blended monthly fee per agent</t>
         </is>
       </c>
       <c r="B21" s="21">
-        <f>IF($B$3="B. Tiered",B8*Scenarios!$E$14+C8*Scenarios!$E$15+D8*Scenarios!$E$16,IF($B$3="A. Flat (current)",B15,B16))</f>
+        <f>IF($B$3="B. Tiered",B6*Scenarios!$E$14+C6*Scenarios!$E$15+D6*Scenarios!$E$16,IF($B$3="D. In-house media",B17,B13))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Share of agents with CRM seat included</t>
-        </is>
-      </c>
-      <c r="B22" s="16">
-        <f>IF($B$3="B. Tiered",C9*Scenarios!$E$15+D9*Scenarios!$E$16,1)</f>
+          <t>Blended transaction fee</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>IF($B$3="B. Tiered",B7*Scenarios!$E$14+C7*Scenarios!$E$15+D7*Scenarios!$E$16,IF($B$3="D. In-house media",B18,B14))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
+          <t>Blended media credit per listing</t>
+        </is>
+      </c>
+      <c r="B23" s="21">
+        <f>IF($B$3="B. Tiered",B8*Scenarios!$E$14+C8*Scenarios!$E$15+D8*Scenarios!$E$16,IF(OR($B$3="A. Flat (current)",$B$3="D. In-house media"),B15,B16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Share of agents with CRM seat included</t>
+        </is>
+      </c>
+      <c r="B24" s="16">
+        <f>IF($B$3="B. Tiered",C9*Scenarios!$E$15+D9*Scenarios!$E$16,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
           <t>Share of transactions with TC included</t>
         </is>
       </c>
-      <c r="B23" s="16">
+      <c r="B25" s="16">
         <f>IF($B$3="B. Tiered",D10*Scenarios!$E$16,0)</f>
         <v/>
       </c>
@@ -1545,7 +1575,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"A. Flat (current),B. Tiered,C. Flat media excluded"</formula1>
+      <formula1>"A. Flat (current),B. Tiered,C. Flat media excluded,D. In-house media"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1558,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1719,7 +1749,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Fixed monthly — the brokerage exists whether or not anyone closes</t>
+          <t>In-house media — you shoot it yourself</t>
         </is>
       </c>
       <c r="B13" s="20" t="n"/>
@@ -1734,33 +1764,37 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Brokerage E&amp;O policy</t>
+          <t>Editing, per listing</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Firm policy. Agents carry their own on top.</t>
+          <t>Your quoted editor rate for photos and video.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>General liability</t>
+          <t>Printed flyers and brochures</t>
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>45</v>
-      </c>
-      <c r="C15" s="12" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Still a print cost whoever shoots it.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Broker association and MLS dues</t>
+          <t>Yard sign and lockbox, amortized</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
@@ -1768,225 +1802,389 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Your own dues, annualized to a month.</t>
+          <t>Unchanged — you are not shooting these.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Website, hosting, domain, email</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C17" s="12" t="inlineStr"/>
+          <t>Your hours per listing</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Drive, shoot interior and exterior, fly the drone, upload, review the edit.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Transaction management platform</t>
+          <t>Value of your hour</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Base tier for a small firm.</t>
+          <t>What an hour of your time is worth doing the next best thing: recruiting an agent or signing a door.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>E-signature</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="n">
-        <v>45</v>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>In-house media, cash cost per listing</t>
+        </is>
+      </c>
+      <c r="B19" s="18">
+        <f>SUM(B14:B16)</f>
+        <v/>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>DocuSign Business Pro is about $45/user/month annually — needed for PowerForms.</t>
+          <t>What actually leaves the bank account.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Accounting and bookkeeping</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n">
-        <v>250</v>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>In-house media, loaded cost per listing</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>B19+B17*B18</f>
+        <v/>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Trust accounting is not a DIY job once agents are closing.</t>
+          <t>Cash plus your time. This is the honest number to price against.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Legal and compliance retainer</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="n">
-        <v>125</v>
+          <t>Listings you can personally shoot per month</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Annual attorney review amortized.</t>
+          <t>Above this, you outsource the overflow at the full package price — or stop taking listings.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Phone system and call routing</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C22" s="12" t="inlineStr"/>
+          <t>Count your time as a cost?</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>1 = yes (recommended). 0 = treat your labor as free and see the flattering version.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Banking, escrow account fees, software</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="C23" s="12" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Marketing and recruiting spend</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n">
-        <v>200</v>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Cards, cap hats, event table fees, boosted posts.</t>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Active media cost per listing</t>
+        </is>
+      </c>
+      <c r="B23" s="18">
+        <f>IF(Tiers!$B$3="D. In-house media",IF(Costs!$B$22=1,Costs!$B$20,Costs!$B$19),Costs!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>What the P&amp;L and unit economics use.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Total fixed monthly</t>
-        </is>
-      </c>
-      <c r="B25" s="18">
-        <f>SUM(B14:B24)</f>
-        <v/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Fixed monthly — the brokerage exists whether or not anyone closes</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Brokerage E&amp;O policy</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Firm policy. Agents carry their own on top.</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>Per agent, per month</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="n"/>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="20" t="n"/>
-      <c r="H27" s="20" t="n"/>
-      <c r="I27" s="20" t="n"/>
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>General liability</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="C27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>CRM seat</t>
+          <t>Broker association and MLS dues</t>
         </is>
       </c>
       <c r="B28" s="17" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Follow Up Boss class tool. Only charged for tiers that include it.</t>
+          <t>Your own dues, annualized to a month.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Email, storage, phone line</t>
+          <t>Website, hosting, domain, email</t>
         </is>
       </c>
       <c r="B29" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>Charged for every agent.</t>
+        <v>35</v>
+      </c>
+      <c r="C29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Transaction management platform</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Base tier for a small firm.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Per transaction</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="20" t="n"/>
-      <c r="F31" s="20" t="n"/>
-      <c r="G31" s="20" t="n"/>
-      <c r="H31" s="20" t="n"/>
-      <c r="I31" s="20" t="n"/>
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>E-signature</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>DocuSign Business Pro is about $45/user/month annually — needed for PowerForms.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Compliance review and file handling</t>
+          <t>Accounting and bookkeeping</t>
         </is>
       </c>
       <c r="B32" s="17" t="n">
-        <v>35</v>
+        <v>250</v>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Your time, costed. It is not free just because you do it.</t>
+          <t>Trust accounting is not a DIY job once agents are closing.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Disbursement and banking</t>
+          <t>Legal and compliance retainer</t>
         </is>
       </c>
       <c r="B33" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="C33" s="12" t="inlineStr"/>
+        <v>125</v>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Annual attorney review amortized.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
+          <t>Phone system and call routing</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="C34" s="12" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Banking, escrow account fees, software</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="C35" s="12" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Marketing and recruiting spend</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Cards, cap hats, event table fees, boosted posts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Total fixed monthly</t>
+        </is>
+      </c>
+      <c r="B37" s="18">
+        <f>SUM(B26:B36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Per agent, per month</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n"/>
+      <c r="C39" s="20" t="n"/>
+      <c r="D39" s="20" t="n"/>
+      <c r="E39" s="20" t="n"/>
+      <c r="F39" s="20" t="n"/>
+      <c r="G39" s="20" t="n"/>
+      <c r="H39" s="20" t="n"/>
+      <c r="I39" s="20" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>CRM seat</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Follow Up Boss class tool. Only charged for tiers that include it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Email, storage, phone line</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Charged for every agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Per transaction</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Compliance review and file handling</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>Your time, costed. It is not free just because you do it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Disbursement and banking</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" s="12" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
           <t>Transaction coordination, when included</t>
         </is>
       </c>
-      <c r="B34" s="17" t="n">
+      <c r="B46" s="17" t="n">
         <v>325</v>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>Outsourced TC per file. Only for tiers that include it.</t>
         </is>
@@ -2003,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2700,99 +2898,99 @@
         </is>
       </c>
       <c r="B13" s="25">
-        <f>B7*Tiers!$B$19</f>
+        <f>B7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="C13" s="25">
-        <f>C7*Tiers!$B$19</f>
+        <f>C7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="D13" s="25">
-        <f>D7*Tiers!$B$19</f>
+        <f>D7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="E13" s="25">
-        <f>E7*Tiers!$B$19</f>
+        <f>E7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="F13" s="25">
-        <f>F7*Tiers!$B$19</f>
+        <f>F7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="G13" s="25">
-        <f>G7*Tiers!$B$19</f>
+        <f>G7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="H13" s="25">
-        <f>H7*Tiers!$B$19</f>
+        <f>H7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="I13" s="25">
-        <f>I7*Tiers!$B$19</f>
+        <f>I7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="J13" s="25">
-        <f>J7*Tiers!$B$19</f>
+        <f>J7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="K13" s="25">
-        <f>K7*Tiers!$B$19</f>
+        <f>K7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="L13" s="25">
-        <f>L7*Tiers!$B$19</f>
+        <f>L7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="M13" s="25">
-        <f>M7*Tiers!$B$19</f>
+        <f>M7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="N13" s="25">
-        <f>N7*Tiers!$B$19</f>
+        <f>N7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="O13" s="25">
-        <f>O7*Tiers!$B$19</f>
+        <f>O7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="P13" s="25">
-        <f>P7*Tiers!$B$19</f>
+        <f>P7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="Q13" s="25">
-        <f>Q7*Tiers!$B$19</f>
+        <f>Q7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="R13" s="25">
-        <f>R7*Tiers!$B$19</f>
+        <f>R7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="S13" s="25">
-        <f>S7*Tiers!$B$19</f>
+        <f>S7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="T13" s="25">
-        <f>T7*Tiers!$B$19</f>
+        <f>T7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="U13" s="25">
-        <f>U7*Tiers!$B$19</f>
+        <f>U7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="V13" s="25">
-        <f>V7*Tiers!$B$19</f>
+        <f>V7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="W13" s="25">
-        <f>W7*Tiers!$B$19</f>
+        <f>W7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="X13" s="25">
-        <f>X7*Tiers!$B$19</f>
+        <f>X7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="Y13" s="25">
-        <f>Y7*Tiers!$B$19</f>
+        <f>Y7*Tiers!$B$21</f>
         <v/>
       </c>
       <c r="Z13" s="18">
@@ -2807,99 +3005,99 @@
         </is>
       </c>
       <c r="B14" s="25">
-        <f>B8*Tiers!$B$20</f>
+        <f>B8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="C14" s="25">
-        <f>C8*Tiers!$B$20</f>
+        <f>C8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>D8*Tiers!$B$20</f>
+        <f>D8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>E8*Tiers!$B$20</f>
+        <f>E8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>F8*Tiers!$B$20</f>
+        <f>F8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="G14" s="25">
-        <f>G8*Tiers!$B$20</f>
+        <f>G8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>H8*Tiers!$B$20</f>
+        <f>H8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="I14" s="25">
-        <f>I8*Tiers!$B$20</f>
+        <f>I8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="J14" s="25">
-        <f>J8*Tiers!$B$20</f>
+        <f>J8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="K14" s="25">
-        <f>K8*Tiers!$B$20</f>
+        <f>K8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="L14" s="25">
-        <f>L8*Tiers!$B$20</f>
+        <f>L8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="M14" s="25">
-        <f>M8*Tiers!$B$20</f>
+        <f>M8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="N14" s="25">
-        <f>N8*Tiers!$B$20</f>
+        <f>N8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="O14" s="25">
-        <f>O8*Tiers!$B$20</f>
+        <f>O8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="P14" s="25">
-        <f>P8*Tiers!$B$20</f>
+        <f>P8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="Q14" s="25">
-        <f>Q8*Tiers!$B$20</f>
+        <f>Q8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="R14" s="25">
-        <f>R8*Tiers!$B$20</f>
+        <f>R8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="S14" s="25">
-        <f>S8*Tiers!$B$20</f>
+        <f>S8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="T14" s="25">
-        <f>T8*Tiers!$B$20</f>
+        <f>T8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="U14" s="25">
-        <f>U8*Tiers!$B$20</f>
+        <f>U8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="V14" s="25">
-        <f>V8*Tiers!$B$20</f>
+        <f>V8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="W14" s="25">
-        <f>W8*Tiers!$B$20</f>
+        <f>W8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="X14" s="25">
-        <f>X8*Tiers!$B$20</f>
+        <f>X8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="Y14" s="25">
-        <f>Y8*Tiers!$B$20</f>
+        <f>Y8*Tiers!$B$22</f>
         <v/>
       </c>
       <c r="Z14" s="18">
@@ -2914,99 +3112,99 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>B10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>B10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>C10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>C10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>D10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>D10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>E10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>E10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>F10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>F10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>G10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>G10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="H15" s="25">
-        <f>H10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>H10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="I15" s="25">
-        <f>I10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>I10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="J15" s="25">
-        <f>J10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>J10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="K15" s="25">
-        <f>K10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>K10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="L15" s="25">
-        <f>L10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>L10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="M15" s="25">
-        <f>M10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>M10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="N15" s="25">
-        <f>N10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>N10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="O15" s="25">
-        <f>O10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>O10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="P15" s="25">
-        <f>P10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>P10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Q15" s="25">
-        <f>Q10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>Q10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="R15" s="25">
-        <f>R10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>R10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="S15" s="25">
-        <f>S10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>S10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="T15" s="25">
-        <f>T10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>T10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="U15" s="25">
-        <f>U10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>U10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="V15" s="25">
-        <f>V10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>V10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="W15" s="25">
-        <f>W10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>W10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="X15" s="25">
-        <f>X10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>X10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Y15" s="25">
-        <f>Y10*MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>Y10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Z15" s="18">
@@ -3139,106 +3337,106 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Media package cost</t>
-        </is>
-      </c>
-      <c r="B19" s="25">
-        <f>B10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="C19" s="25">
-        <f>C10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="D19" s="25">
-        <f>D10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="E19" s="25">
-        <f>E10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="F19" s="25">
-        <f>F10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="G19" s="25">
-        <f>G10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="H19" s="25">
-        <f>H10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="I19" s="25">
-        <f>I10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="J19" s="25">
-        <f>J10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="K19" s="25">
-        <f>K10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="L19" s="25">
-        <f>L10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="M19" s="25">
-        <f>M10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="N19" s="25">
-        <f>N10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="O19" s="25">
-        <f>O10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="P19" s="25">
-        <f>P10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Q19" s="25">
-        <f>Q10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="R19" s="25">
-        <f>R10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="S19" s="25">
-        <f>S10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="T19" s="25">
-        <f>T10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="U19" s="25">
-        <f>U10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="V19" s="25">
-        <f>V10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="W19" s="25">
-        <f>W10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="X19" s="25">
-        <f>X10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Y19" s="25">
-        <f>Y10*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Z19" s="18">
+          <t>Listings above your shooting capacity</t>
+        </is>
+      </c>
+      <c r="B19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,B10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="C19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,C10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="D19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,D10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,E10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,F10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,G10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="H19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,H10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="I19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,I10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="J19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,J10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="K19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,K10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="L19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,L10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,M10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="N19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,N10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="O19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,O10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,P10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Q10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="R19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,R10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="S19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,S10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="T19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,T10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="U19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,U10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="V19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,V10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="W19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,W10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="X19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,X10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="Y19" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Y10-Costs!$B$21),0)</f>
+        <v/>
+      </c>
+      <c r="Z19" s="14">
         <f>SUM(B19:Y19)</f>
         <v/>
       </c>
@@ -3246,103 +3444,103 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Per-transaction cost</t>
+          <t>Media cost</t>
         </is>
       </c>
       <c r="B20" s="25">
-        <f>B8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(B10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,B10))*Costs!$B$23+B19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>C8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(C10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,C10))*Costs!$B$23+C19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="D20" s="25">
-        <f>D8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(D10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,D10))*Costs!$B$23+D19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="E20" s="25">
-        <f>E8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(E10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,E10))*Costs!$B$23+E19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="F20" s="25">
-        <f>F8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(F10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,F10))*Costs!$B$23+F19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="G20" s="25">
-        <f>G8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(G10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,G10))*Costs!$B$23+G19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="H20" s="25">
-        <f>H8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(H10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,H10))*Costs!$B$23+H19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="I20" s="25">
-        <f>I8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(I10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,I10))*Costs!$B$23+I19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="J20" s="25">
-        <f>J8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(J10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,J10))*Costs!$B$23+J19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="K20" s="25">
-        <f>K8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(K10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,K10))*Costs!$B$23+K19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="L20" s="25">
-        <f>L8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(L10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,L10))*Costs!$B$23+L19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="M20" s="25">
-        <f>M8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(M10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,M10))*Costs!$B$23+M19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="N20" s="25">
-        <f>N8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(N10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,N10))*Costs!$B$23+N19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="O20" s="25">
-        <f>O8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(O10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,O10))*Costs!$B$23+O19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="P20" s="25">
-        <f>P8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(P10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,P10))*Costs!$B$23+P19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Q20" s="25">
-        <f>Q8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(Q10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,Q10))*Costs!$B$23+Q19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="R20" s="25">
-        <f>R8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(R10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,R10))*Costs!$B$23+R19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="S20" s="25">
-        <f>S8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(S10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,S10))*Costs!$B$23+S19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="T20" s="25">
-        <f>T8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(T10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,T10))*Costs!$B$23+T19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="U20" s="25">
-        <f>U8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(U10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,U10))*Costs!$B$23+U19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="V20" s="25">
-        <f>V8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(V10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,V10))*Costs!$B$23+V19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="W20" s="25">
-        <f>W8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(W10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,W10))*Costs!$B$23+W19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="X20" s="25">
-        <f>X8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(X10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,X10))*Costs!$B$23+X19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Y20" s="25">
-        <f>Y8*((Costs!$B$32+Costs!$B$33)+Tiers!$B$23*Costs!$B$34)</f>
+        <f>MIN(Y10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,Y10))*Costs!$B$23+Y19*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Z20" s="18">
@@ -3353,103 +3551,103 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Per-agent cost</t>
+          <t>Per-transaction cost</t>
         </is>
       </c>
       <c r="B21" s="25">
-        <f>B7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>B8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>C7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>C8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>D7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>D8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="E21" s="25">
-        <f>E7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>E8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="F21" s="25">
-        <f>F7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>F8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="G21" s="25">
-        <f>G7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>G8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="H21" s="25">
-        <f>H7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>H8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="I21" s="25">
-        <f>I7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>I8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="J21" s="25">
-        <f>J7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>J8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="K21" s="25">
-        <f>K7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>K8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="L21" s="25">
-        <f>L7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>L8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="M21" s="25">
-        <f>M7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>M8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="N21" s="25">
-        <f>N7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>N8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="O21" s="25">
-        <f>O7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>O8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="P21" s="25">
-        <f>P7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>P8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Q21" s="25">
-        <f>Q7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>Q8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="R21" s="25">
-        <f>R7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>R8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="S21" s="25">
-        <f>S7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>S8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="T21" s="25">
-        <f>T7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>T8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="U21" s="25">
-        <f>U7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>U8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="V21" s="25">
-        <f>V7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>V8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="W21" s="25">
-        <f>W7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>W8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="X21" s="25">
-        <f>X7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>X8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Y21" s="25">
-        <f>Y7*(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>Y8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Z21" s="18">
@@ -3460,103 +3658,103 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Fixed overhead</t>
+          <t>Per-agent cost</t>
         </is>
       </c>
       <c r="B22" s="25">
-        <f>Costs!$B$25</f>
+        <f>B7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>Costs!$B$25</f>
+        <f>C7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="D22" s="25">
-        <f>Costs!$B$25</f>
+        <f>D7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="E22" s="25">
-        <f>Costs!$B$25</f>
+        <f>E7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="F22" s="25">
-        <f>Costs!$B$25</f>
+        <f>F7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="G22" s="25">
-        <f>Costs!$B$25</f>
+        <f>G7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="H22" s="25">
-        <f>Costs!$B$25</f>
+        <f>H7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="I22" s="25">
-        <f>Costs!$B$25</f>
+        <f>I7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="J22" s="25">
-        <f>Costs!$B$25</f>
+        <f>J7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="K22" s="25">
-        <f>Costs!$B$25</f>
+        <f>K7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="L22" s="25">
-        <f>Costs!$B$25</f>
+        <f>L7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="M22" s="25">
-        <f>Costs!$B$25</f>
+        <f>M7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="N22" s="25">
-        <f>Costs!$B$25</f>
+        <f>N7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="O22" s="25">
-        <f>Costs!$B$25</f>
+        <f>O7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="P22" s="25">
-        <f>Costs!$B$25</f>
+        <f>P7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="Q22" s="25">
-        <f>Costs!$B$25</f>
+        <f>Q7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="R22" s="25">
-        <f>Costs!$B$25</f>
+        <f>R7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="S22" s="25">
-        <f>Costs!$B$25</f>
+        <f>S7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="T22" s="25">
-        <f>Costs!$B$25</f>
+        <f>T7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="U22" s="25">
-        <f>Costs!$B$25</f>
+        <f>U7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="V22" s="25">
-        <f>Costs!$B$25</f>
+        <f>V7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="W22" s="25">
-        <f>Costs!$B$25</f>
+        <f>W7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="X22" s="25">
-        <f>Costs!$B$25</f>
+        <f>X7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="Y22" s="25">
-        <f>Costs!$B$25</f>
+        <f>Y7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
       <c r="Z22" s="18">
@@ -3567,103 +3765,103 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Managing agent compensation</t>
+          <t>Fixed overhead</t>
         </is>
       </c>
       <c r="B23" s="25">
-        <f>'Managing Agent'!B$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>'Managing Agent'!C$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="D23" s="25">
-        <f>'Managing Agent'!D$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="E23" s="25">
-        <f>'Managing Agent'!E$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="F23" s="25">
-        <f>'Managing Agent'!F$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="G23" s="25">
-        <f>'Managing Agent'!G$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="H23" s="25">
-        <f>'Managing Agent'!H$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="I23" s="25">
-        <f>'Managing Agent'!I$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="J23" s="25">
-        <f>'Managing Agent'!J$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="K23" s="25">
-        <f>'Managing Agent'!K$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="L23" s="25">
-        <f>'Managing Agent'!L$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="M23" s="25">
-        <f>'Managing Agent'!M$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="N23" s="25">
-        <f>'Managing Agent'!N$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="O23" s="25">
-        <f>'Managing Agent'!O$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="P23" s="25">
-        <f>'Managing Agent'!P$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="Q23" s="25">
-        <f>'Managing Agent'!Q$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="R23" s="25">
-        <f>'Managing Agent'!R$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="S23" s="25">
-        <f>'Managing Agent'!S$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="T23" s="25">
-        <f>'Managing Agent'!T$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="U23" s="25">
-        <f>'Managing Agent'!U$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="V23" s="25">
-        <f>'Managing Agent'!V$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="W23" s="25">
-        <f>'Managing Agent'!W$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="X23" s="25">
-        <f>'Managing Agent'!X$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="Y23" s="25">
-        <f>'Managing Agent'!Y$30</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
       <c r="Z23" s="18">
@@ -3672,105 +3870,105 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Total cost</t>
-        </is>
-      </c>
-      <c r="B24" s="18">
-        <f>SUM(B19:B23)</f>
-        <v/>
-      </c>
-      <c r="C24" s="18">
-        <f>SUM(C19:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="18">
-        <f>SUM(D19:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="18">
-        <f>SUM(E19:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="18">
-        <f>SUM(F19:F23)</f>
-        <v/>
-      </c>
-      <c r="G24" s="18">
-        <f>SUM(G19:G23)</f>
-        <v/>
-      </c>
-      <c r="H24" s="18">
-        <f>SUM(H19:H23)</f>
-        <v/>
-      </c>
-      <c r="I24" s="18">
-        <f>SUM(I19:I23)</f>
-        <v/>
-      </c>
-      <c r="J24" s="18">
-        <f>SUM(J19:J23)</f>
-        <v/>
-      </c>
-      <c r="K24" s="18">
-        <f>SUM(K19:K23)</f>
-        <v/>
-      </c>
-      <c r="L24" s="18">
-        <f>SUM(L19:L23)</f>
-        <v/>
-      </c>
-      <c r="M24" s="18">
-        <f>SUM(M19:M23)</f>
-        <v/>
-      </c>
-      <c r="N24" s="18">
-        <f>SUM(N19:N23)</f>
-        <v/>
-      </c>
-      <c r="O24" s="18">
-        <f>SUM(O19:O23)</f>
-        <v/>
-      </c>
-      <c r="P24" s="18">
-        <f>SUM(P19:P23)</f>
-        <v/>
-      </c>
-      <c r="Q24" s="18">
-        <f>SUM(Q19:Q23)</f>
-        <v/>
-      </c>
-      <c r="R24" s="18">
-        <f>SUM(R19:R23)</f>
-        <v/>
-      </c>
-      <c r="S24" s="18">
-        <f>SUM(S19:S23)</f>
-        <v/>
-      </c>
-      <c r="T24" s="18">
-        <f>SUM(T19:T23)</f>
-        <v/>
-      </c>
-      <c r="U24" s="18">
-        <f>SUM(U19:U23)</f>
-        <v/>
-      </c>
-      <c r="V24" s="18">
-        <f>SUM(V19:V23)</f>
-        <v/>
-      </c>
-      <c r="W24" s="18">
-        <f>SUM(W19:W23)</f>
-        <v/>
-      </c>
-      <c r="X24" s="18">
-        <f>SUM(X19:X23)</f>
-        <v/>
-      </c>
-      <c r="Y24" s="18">
-        <f>SUM(Y19:Y23)</f>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Managing agent compensation</t>
+        </is>
+      </c>
+      <c r="B24" s="25">
+        <f>'Managing Agent'!B$30</f>
+        <v/>
+      </c>
+      <c r="C24" s="25">
+        <f>'Managing Agent'!C$30</f>
+        <v/>
+      </c>
+      <c r="D24" s="25">
+        <f>'Managing Agent'!D$30</f>
+        <v/>
+      </c>
+      <c r="E24" s="25">
+        <f>'Managing Agent'!E$30</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>'Managing Agent'!F$30</f>
+        <v/>
+      </c>
+      <c r="G24" s="25">
+        <f>'Managing Agent'!G$30</f>
+        <v/>
+      </c>
+      <c r="H24" s="25">
+        <f>'Managing Agent'!H$30</f>
+        <v/>
+      </c>
+      <c r="I24" s="25">
+        <f>'Managing Agent'!I$30</f>
+        <v/>
+      </c>
+      <c r="J24" s="25">
+        <f>'Managing Agent'!J$30</f>
+        <v/>
+      </c>
+      <c r="K24" s="25">
+        <f>'Managing Agent'!K$30</f>
+        <v/>
+      </c>
+      <c r="L24" s="25">
+        <f>'Managing Agent'!L$30</f>
+        <v/>
+      </c>
+      <c r="M24" s="25">
+        <f>'Managing Agent'!M$30</f>
+        <v/>
+      </c>
+      <c r="N24" s="25">
+        <f>'Managing Agent'!N$30</f>
+        <v/>
+      </c>
+      <c r="O24" s="25">
+        <f>'Managing Agent'!O$30</f>
+        <v/>
+      </c>
+      <c r="P24" s="25">
+        <f>'Managing Agent'!P$30</f>
+        <v/>
+      </c>
+      <c r="Q24" s="25">
+        <f>'Managing Agent'!Q$30</f>
+        <v/>
+      </c>
+      <c r="R24" s="25">
+        <f>'Managing Agent'!R$30</f>
+        <v/>
+      </c>
+      <c r="S24" s="25">
+        <f>'Managing Agent'!S$30</f>
+        <v/>
+      </c>
+      <c r="T24" s="25">
+        <f>'Managing Agent'!T$30</f>
+        <v/>
+      </c>
+      <c r="U24" s="25">
+        <f>'Managing Agent'!U$30</f>
+        <v/>
+      </c>
+      <c r="V24" s="25">
+        <f>'Managing Agent'!V$30</f>
+        <v/>
+      </c>
+      <c r="W24" s="25">
+        <f>'Managing Agent'!W$30</f>
+        <v/>
+      </c>
+      <c r="X24" s="25">
+        <f>'Managing Agent'!X$30</f>
+        <v/>
+      </c>
+      <c r="Y24" s="25">
+        <f>'Managing Agent'!Y$30</f>
         <v/>
       </c>
       <c r="Z24" s="18">
@@ -3778,324 +3976,431 @@
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B26" s="18">
-        <f>B16-B24</f>
-        <v/>
-      </c>
-      <c r="C26" s="18">
-        <f>C16-C24</f>
-        <v/>
-      </c>
-      <c r="D26" s="18">
-        <f>D16-D24</f>
-        <v/>
-      </c>
-      <c r="E26" s="18">
-        <f>E16-E24</f>
-        <v/>
-      </c>
-      <c r="F26" s="18">
-        <f>F16-F24</f>
-        <v/>
-      </c>
-      <c r="G26" s="18">
-        <f>G16-G24</f>
-        <v/>
-      </c>
-      <c r="H26" s="18">
-        <f>H16-H24</f>
-        <v/>
-      </c>
-      <c r="I26" s="18">
-        <f>I16-I24</f>
-        <v/>
-      </c>
-      <c r="J26" s="18">
-        <f>J16-J24</f>
-        <v/>
-      </c>
-      <c r="K26" s="18">
-        <f>K16-K24</f>
-        <v/>
-      </c>
-      <c r="L26" s="18">
-        <f>L16-L24</f>
-        <v/>
-      </c>
-      <c r="M26" s="18">
-        <f>M16-M24</f>
-        <v/>
-      </c>
-      <c r="N26" s="18">
-        <f>N16-N24</f>
-        <v/>
-      </c>
-      <c r="O26" s="18">
-        <f>O16-O24</f>
-        <v/>
-      </c>
-      <c r="P26" s="18">
-        <f>P16-P24</f>
-        <v/>
-      </c>
-      <c r="Q26" s="18">
-        <f>Q16-Q24</f>
-        <v/>
-      </c>
-      <c r="R26" s="18">
-        <f>R16-R24</f>
-        <v/>
-      </c>
-      <c r="S26" s="18">
-        <f>S16-S24</f>
-        <v/>
-      </c>
-      <c r="T26" s="18">
-        <f>T16-T24</f>
-        <v/>
-      </c>
-      <c r="U26" s="18">
-        <f>U16-U24</f>
-        <v/>
-      </c>
-      <c r="V26" s="18">
-        <f>V16-V24</f>
-        <v/>
-      </c>
-      <c r="W26" s="18">
-        <f>W16-W24</f>
-        <v/>
-      </c>
-      <c r="X26" s="18">
-        <f>X16-X24</f>
-        <v/>
-      </c>
-      <c r="Y26" s="18">
-        <f>Y16-Y24</f>
-        <v/>
-      </c>
-      <c r="Z26" s="18">
-        <f>SUM(B26:Y26)</f>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Total cost</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>SUM(B20:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="18">
+        <f>SUM(C20:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="18">
+        <f>SUM(D20:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="18">
+        <f>SUM(E20:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="18">
+        <f>SUM(F20:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="18">
+        <f>SUM(G20:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="18">
+        <f>SUM(H20:H24)</f>
+        <v/>
+      </c>
+      <c r="I25" s="18">
+        <f>SUM(I20:I24)</f>
+        <v/>
+      </c>
+      <c r="J25" s="18">
+        <f>SUM(J20:J24)</f>
+        <v/>
+      </c>
+      <c r="K25" s="18">
+        <f>SUM(K20:K24)</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>SUM(L20:L24)</f>
+        <v/>
+      </c>
+      <c r="M25" s="18">
+        <f>SUM(M20:M24)</f>
+        <v/>
+      </c>
+      <c r="N25" s="18">
+        <f>SUM(N20:N24)</f>
+        <v/>
+      </c>
+      <c r="O25" s="18">
+        <f>SUM(O20:O24)</f>
+        <v/>
+      </c>
+      <c r="P25" s="18">
+        <f>SUM(P20:P24)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="18">
+        <f>SUM(Q20:Q24)</f>
+        <v/>
+      </c>
+      <c r="R25" s="18">
+        <f>SUM(R20:R24)</f>
+        <v/>
+      </c>
+      <c r="S25" s="18">
+        <f>SUM(S20:S24)</f>
+        <v/>
+      </c>
+      <c r="T25" s="18">
+        <f>SUM(T20:T24)</f>
+        <v/>
+      </c>
+      <c r="U25" s="18">
+        <f>SUM(U20:U24)</f>
+        <v/>
+      </c>
+      <c r="V25" s="18">
+        <f>SUM(V20:V24)</f>
+        <v/>
+      </c>
+      <c r="W25" s="18">
+        <f>SUM(W20:W24)</f>
+        <v/>
+      </c>
+      <c r="X25" s="18">
+        <f>SUM(X20:X24)</f>
+        <v/>
+      </c>
+      <c r="Y25" s="18">
+        <f>SUM(Y20:Y24)</f>
+        <v/>
+      </c>
+      <c r="Z25" s="18">
+        <f>SUM(B25:Y25)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B27" s="18">
+        <f>B16-B25</f>
+        <v/>
+      </c>
+      <c r="C27" s="18">
+        <f>C16-C25</f>
+        <v/>
+      </c>
+      <c r="D27" s="18">
+        <f>D16-D25</f>
+        <v/>
+      </c>
+      <c r="E27" s="18">
+        <f>E16-E25</f>
+        <v/>
+      </c>
+      <c r="F27" s="18">
+        <f>F16-F25</f>
+        <v/>
+      </c>
+      <c r="G27" s="18">
+        <f>G16-G25</f>
+        <v/>
+      </c>
+      <c r="H27" s="18">
+        <f>H16-H25</f>
+        <v/>
+      </c>
+      <c r="I27" s="18">
+        <f>I16-I25</f>
+        <v/>
+      </c>
+      <c r="J27" s="18">
+        <f>J16-J25</f>
+        <v/>
+      </c>
+      <c r="K27" s="18">
+        <f>K16-K25</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>L16-L25</f>
+        <v/>
+      </c>
+      <c r="M27" s="18">
+        <f>M16-M25</f>
+        <v/>
+      </c>
+      <c r="N27" s="18">
+        <f>N16-N25</f>
+        <v/>
+      </c>
+      <c r="O27" s="18">
+        <f>O16-O25</f>
+        <v/>
+      </c>
+      <c r="P27" s="18">
+        <f>P16-P25</f>
+        <v/>
+      </c>
+      <c r="Q27" s="18">
+        <f>Q16-Q25</f>
+        <v/>
+      </c>
+      <c r="R27" s="18">
+        <f>R16-R25</f>
+        <v/>
+      </c>
+      <c r="S27" s="18">
+        <f>S16-S25</f>
+        <v/>
+      </c>
+      <c r="T27" s="18">
+        <f>T16-T25</f>
+        <v/>
+      </c>
+      <c r="U27" s="18">
+        <f>U16-U25</f>
+        <v/>
+      </c>
+      <c r="V27" s="18">
+        <f>V16-V25</f>
+        <v/>
+      </c>
+      <c r="W27" s="18">
+        <f>W16-W25</f>
+        <v/>
+      </c>
+      <c r="X27" s="18">
+        <f>X16-X25</f>
+        <v/>
+      </c>
+      <c r="Y27" s="18">
+        <f>Y16-Y25</f>
+        <v/>
+      </c>
+      <c r="Z27" s="18">
+        <f>SUM(B27:Y27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>Cumulative EBITDA</t>
         </is>
       </c>
-      <c r="B27" s="18">
-        <f>B26</f>
-        <v/>
-      </c>
-      <c r="C27" s="18">
-        <f>B27+C26</f>
-        <v/>
-      </c>
-      <c r="D27" s="18">
-        <f>C27+D26</f>
-        <v/>
-      </c>
-      <c r="E27" s="18">
-        <f>D27+E26</f>
-        <v/>
-      </c>
-      <c r="F27" s="18">
-        <f>E27+F26</f>
-        <v/>
-      </c>
-      <c r="G27" s="18">
-        <f>F27+G26</f>
-        <v/>
-      </c>
-      <c r="H27" s="18">
-        <f>G27+H26</f>
-        <v/>
-      </c>
-      <c r="I27" s="18">
-        <f>H27+I26</f>
-        <v/>
-      </c>
-      <c r="J27" s="18">
-        <f>I27+J26</f>
-        <v/>
-      </c>
-      <c r="K27" s="18">
-        <f>J27+K26</f>
-        <v/>
-      </c>
-      <c r="L27" s="18">
-        <f>K27+L26</f>
-        <v/>
-      </c>
-      <c r="M27" s="18">
-        <f>L27+M26</f>
-        <v/>
-      </c>
-      <c r="N27" s="18">
-        <f>M27+N26</f>
-        <v/>
-      </c>
-      <c r="O27" s="18">
-        <f>N27+O26</f>
-        <v/>
-      </c>
-      <c r="P27" s="18">
-        <f>O27+P26</f>
-        <v/>
-      </c>
-      <c r="Q27" s="18">
-        <f>P27+Q26</f>
-        <v/>
-      </c>
-      <c r="R27" s="18">
-        <f>Q27+R26</f>
-        <v/>
-      </c>
-      <c r="S27" s="18">
-        <f>R27+S26</f>
-        <v/>
-      </c>
-      <c r="T27" s="18">
-        <f>S27+T26</f>
-        <v/>
-      </c>
-      <c r="U27" s="18">
-        <f>T27+U26</f>
-        <v/>
-      </c>
-      <c r="V27" s="18">
-        <f>U27+V26</f>
-        <v/>
-      </c>
-      <c r="W27" s="18">
-        <f>V27+W26</f>
-        <v/>
-      </c>
-      <c r="X27" s="18">
-        <f>W27+X26</f>
-        <v/>
-      </c>
-      <c r="Y27" s="18">
-        <f>X27+Y26</f>
-        <v/>
-      </c>
-      <c r="Z27" s="18">
-        <f>Y27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="B28" s="18">
+        <f>B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="18">
+        <f>B28+C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="18">
+        <f>C28+D27</f>
+        <v/>
+      </c>
+      <c r="E28" s="18">
+        <f>D28+E27</f>
+        <v/>
+      </c>
+      <c r="F28" s="18">
+        <f>E28+F27</f>
+        <v/>
+      </c>
+      <c r="G28" s="18">
+        <f>F28+G27</f>
+        <v/>
+      </c>
+      <c r="H28" s="18">
+        <f>G28+H27</f>
+        <v/>
+      </c>
+      <c r="I28" s="18">
+        <f>H28+I27</f>
+        <v/>
+      </c>
+      <c r="J28" s="18">
+        <f>I28+J27</f>
+        <v/>
+      </c>
+      <c r="K28" s="18">
+        <f>J28+K27</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>K28+L27</f>
+        <v/>
+      </c>
+      <c r="M28" s="18">
+        <f>L28+M27</f>
+        <v/>
+      </c>
+      <c r="N28" s="18">
+        <f>M28+N27</f>
+        <v/>
+      </c>
+      <c r="O28" s="18">
+        <f>N28+O27</f>
+        <v/>
+      </c>
+      <c r="P28" s="18">
+        <f>O28+P27</f>
+        <v/>
+      </c>
+      <c r="Q28" s="18">
+        <f>P28+Q27</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>Q28+R27</f>
+        <v/>
+      </c>
+      <c r="S28" s="18">
+        <f>R28+S27</f>
+        <v/>
+      </c>
+      <c r="T28" s="18">
+        <f>S28+T27</f>
+        <v/>
+      </c>
+      <c r="U28" s="18">
+        <f>T28+U27</f>
+        <v/>
+      </c>
+      <c r="V28" s="18">
+        <f>U28+V27</f>
+        <v/>
+      </c>
+      <c r="W28" s="18">
+        <f>V28+W27</f>
+        <v/>
+      </c>
+      <c r="X28" s="18">
+        <f>W28+X27</f>
+        <v/>
+      </c>
+      <c r="Y28" s="18">
+        <f>X28+Y27</f>
+        <v/>
+      </c>
+      <c r="Z28" s="18">
+        <f>Y28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
       </c>
-      <c r="B28" s="26">
-        <f>IFERROR(B26/B16,0)</f>
-        <v/>
-      </c>
-      <c r="C28" s="26">
-        <f>IFERROR(C26/C16,0)</f>
-        <v/>
-      </c>
-      <c r="D28" s="26">
-        <f>IFERROR(D26/D16,0)</f>
-        <v/>
-      </c>
-      <c r="E28" s="26">
-        <f>IFERROR(E26/E16,0)</f>
-        <v/>
-      </c>
-      <c r="F28" s="26">
-        <f>IFERROR(F26/F16,0)</f>
-        <v/>
-      </c>
-      <c r="G28" s="26">
-        <f>IFERROR(G26/G16,0)</f>
-        <v/>
-      </c>
-      <c r="H28" s="26">
-        <f>IFERROR(H26/H16,0)</f>
-        <v/>
-      </c>
-      <c r="I28" s="26">
-        <f>IFERROR(I26/I16,0)</f>
-        <v/>
-      </c>
-      <c r="J28" s="26">
-        <f>IFERROR(J26/J16,0)</f>
-        <v/>
-      </c>
-      <c r="K28" s="26">
-        <f>IFERROR(K26/K16,0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="26">
-        <f>IFERROR(L26/L16,0)</f>
-        <v/>
-      </c>
-      <c r="M28" s="26">
-        <f>IFERROR(M26/M16,0)</f>
-        <v/>
-      </c>
-      <c r="N28" s="26">
-        <f>IFERROR(N26/N16,0)</f>
-        <v/>
-      </c>
-      <c r="O28" s="26">
-        <f>IFERROR(O26/O16,0)</f>
-        <v/>
-      </c>
-      <c r="P28" s="26">
-        <f>IFERROR(P26/P16,0)</f>
-        <v/>
-      </c>
-      <c r="Q28" s="26">
-        <f>IFERROR(Q26/Q16,0)</f>
-        <v/>
-      </c>
-      <c r="R28" s="26">
-        <f>IFERROR(R26/R16,0)</f>
-        <v/>
-      </c>
-      <c r="S28" s="26">
-        <f>IFERROR(S26/S16,0)</f>
-        <v/>
-      </c>
-      <c r="T28" s="26">
-        <f>IFERROR(T26/T16,0)</f>
-        <v/>
-      </c>
-      <c r="U28" s="26">
-        <f>IFERROR(U26/U16,0)</f>
-        <v/>
-      </c>
-      <c r="V28" s="26">
-        <f>IFERROR(V26/V16,0)</f>
-        <v/>
-      </c>
-      <c r="W28" s="26">
-        <f>IFERROR(W26/W16,0)</f>
-        <v/>
-      </c>
-      <c r="X28" s="26">
-        <f>IFERROR(X26/X16,0)</f>
-        <v/>
-      </c>
-      <c r="Y28" s="26">
-        <f>IFERROR(Y26/Y16,0)</f>
-        <v/>
-      </c>
-      <c r="Z28" s="16">
-        <f>IFERROR(Z26/Z16,0)</f>
+      <c r="B29" s="26">
+        <f>IFERROR(B27/B16,0)</f>
+        <v/>
+      </c>
+      <c r="C29" s="26">
+        <f>IFERROR(C27/C16,0)</f>
+        <v/>
+      </c>
+      <c r="D29" s="26">
+        <f>IFERROR(D27/D16,0)</f>
+        <v/>
+      </c>
+      <c r="E29" s="26">
+        <f>IFERROR(E27/E16,0)</f>
+        <v/>
+      </c>
+      <c r="F29" s="26">
+        <f>IFERROR(F27/F16,0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="26">
+        <f>IFERROR(G27/G16,0)</f>
+        <v/>
+      </c>
+      <c r="H29" s="26">
+        <f>IFERROR(H27/H16,0)</f>
+        <v/>
+      </c>
+      <c r="I29" s="26">
+        <f>IFERROR(I27/I16,0)</f>
+        <v/>
+      </c>
+      <c r="J29" s="26">
+        <f>IFERROR(J27/J16,0)</f>
+        <v/>
+      </c>
+      <c r="K29" s="26">
+        <f>IFERROR(K27/K16,0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="26">
+        <f>IFERROR(L27/L16,0)</f>
+        <v/>
+      </c>
+      <c r="M29" s="26">
+        <f>IFERROR(M27/M16,0)</f>
+        <v/>
+      </c>
+      <c r="N29" s="26">
+        <f>IFERROR(N27/N16,0)</f>
+        <v/>
+      </c>
+      <c r="O29" s="26">
+        <f>IFERROR(O27/O16,0)</f>
+        <v/>
+      </c>
+      <c r="P29" s="26">
+        <f>IFERROR(P27/P16,0)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="26">
+        <f>IFERROR(Q27/Q16,0)</f>
+        <v/>
+      </c>
+      <c r="R29" s="26">
+        <f>IFERROR(R27/R16,0)</f>
+        <v/>
+      </c>
+      <c r="S29" s="26">
+        <f>IFERROR(S27/S16,0)</f>
+        <v/>
+      </c>
+      <c r="T29" s="26">
+        <f>IFERROR(T27/T16,0)</f>
+        <v/>
+      </c>
+      <c r="U29" s="26">
+        <f>IFERROR(U27/U16,0)</f>
+        <v/>
+      </c>
+      <c r="V29" s="26">
+        <f>IFERROR(V27/V16,0)</f>
+        <v/>
+      </c>
+      <c r="W29" s="26">
+        <f>IFERROR(W27/W16,0)</f>
+        <v/>
+      </c>
+      <c r="X29" s="26">
+        <f>IFERROR(X27/X16,0)</f>
+        <v/>
+      </c>
+      <c r="Y29" s="26">
+        <f>IFERROR(Y27/Y16,0)</f>
+        <v/>
+      </c>
+      <c r="Z29" s="16">
+        <f>IFERROR(Z27/Z16,0)</f>
         <v/>
       </c>
     </row>
@@ -4155,7 +4460,7 @@
         </is>
       </c>
       <c r="B4" s="27">
-        <f>Tiers!$B$20</f>
+        <f>Tiers!$B$22</f>
         <v/>
       </c>
     </row>
@@ -4166,7 +4471,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>-(Costs!$B$32+Costs!$B$33)</f>
+        <f>-(Costs!$B$44+Costs!$B$45)</f>
         <v/>
       </c>
     </row>
@@ -4177,7 +4482,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>-Tiers!$B$23*Costs!$B$34</f>
+        <f>-Tiers!$B$25*Costs!$B$46</f>
         <v/>
       </c>
     </row>
@@ -4205,7 +4510,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>-Costs!$B$11</f>
+        <f>-Costs!$B$23</f>
         <v/>
       </c>
     </row>
@@ -4216,7 +4521,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>MAX(0,Costs!$B$11-Tiers!$B$21)</f>
+        <f>MAX(0,Costs!$B$23-Tiers!$B$23)</f>
         <v/>
       </c>
     </row>
@@ -4269,7 +4574,7 @@
         </is>
       </c>
       <c r="B16" s="27">
-        <f>Tiers!$B$19</f>
+        <f>Tiers!$B$21</f>
         <v/>
       </c>
     </row>
@@ -4280,7 +4585,7 @@
         </is>
       </c>
       <c r="B17" s="27">
-        <f>-(Costs!$B$29+Tiers!$B$22*Costs!$B$28)</f>
+        <f>-(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
         <v/>
       </c>
     </row>
@@ -4339,7 +4644,7 @@
         </is>
       </c>
       <c r="B23" s="28">
-        <f>Costs!$B$25</f>
+        <f>Costs!$B$37</f>
         <v/>
       </c>
     </row>
@@ -5479,7 +5784,7 @@
         </is>
       </c>
       <c r="B36" s="18">
-        <f>-(12*Tiers!$B$19+B33*12*Tiers!$B$20)</f>
+        <f>-(12*Tiers!$B$21+B33*12*Tiers!$B$22)</f>
         <v/>
       </c>
     </row>
@@ -5712,7 +6017,7 @@
         </is>
       </c>
       <c r="B16" s="28">
-        <f>SUM('P&amp;L'!N26:Y26)</f>
+        <f>SUM('P&amp;L'!N27:Y27)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Media is editing only; flyers and signage become priced add-ons
Brokerage absorbs the $65 edit per listing. Flyers ($60) and sign/lockbox ($85)
move to an add-on block sold at cost plus a markup, with attach rates.

Effect at $399 + $99/month, modest case: listing contribution goes from -$42 to
+$116, break-even from 12 agents to 9, year-2 EBITDA from $13.4k to $21.8k.

The 10% markup earns $12.88 per listing. It is a convenience for the agent, not
a profit centre, and the model labels it that way.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -1588,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1772,419 +1772,487 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Your quoted editor rate for photos and video.</t>
+          <t>Your quoted editor rate for photos and video. The only media cost the brokerage absorbs.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Printed flyers and brochures</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n">
-        <v>60</v>
+          <t>Your hours per listing</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>2.5</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Still a print cost whoever shoots it.</t>
+          <t>Drive, shoot interior and exterior, fly the drone, upload, review the edit.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Yard sign and lockbox, amortized</t>
+          <t>Value of your hour</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Unchanged — you are not shooting these.</t>
+          <t>What an hour of your time is worth doing the next best thing: recruiting an agent or signing a door.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Your hours per listing</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>2.5</v>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>In-house media, cash cost per listing</t>
+        </is>
+      </c>
+      <c r="B17" s="18">
+        <f>B14</f>
+        <v/>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Drive, shoot interior and exterior, fly the drone, upload, review the edit.</t>
+          <t>What actually leaves the bank account.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>Value of your hour</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n">
-        <v>75</v>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>In-house media, loaded cost per listing</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>B17+B15*B16</f>
+        <v/>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>What an hour of your time is worth doing the next best thing: recruiting an agent or signing a door.</t>
+          <t>Cash plus your time. This is the honest number to price against.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>In-house media, cash cost per listing</t>
-        </is>
-      </c>
-      <c r="B19" s="18">
-        <f>SUM(B14:B16)</f>
-        <v/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Listings you can personally shoot per month</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>What actually leaves the bank account.</t>
+          <t>Above this, you outsource the overflow at the full package price — or stop taking listings.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>In-house media, loaded cost per listing</t>
-        </is>
-      </c>
-      <c r="B20" s="18">
-        <f>B19+B17*B18</f>
-        <v/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Count your time as a cost?</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Cash plus your time. This is the honest number to price against.</t>
+          <t>1 = yes (recommended). 0 = treat your labor as free and see the flattering version.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Listings you can personally shoot per month</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Above this, you outsource the overflow at the full package price — or stop taking listings.</t>
-        </is>
-      </c>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Add-ons sold to the agent at cost plus a markup</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="20" t="n"/>
+      <c r="D21" s="20" t="n"/>
+      <c r="E21" s="20" t="n"/>
+      <c r="F21" s="20" t="n"/>
+      <c r="G21" s="20" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Count your time as a cost?</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>1</v>
+          <t>Printed flyers and brochures — cost</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>60</v>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>1 = yes (recommended). 0 = treat your labor as free and see the flattering version.</t>
+          <t>Short run, per listing.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Active media cost per listing</t>
-        </is>
-      </c>
-      <c r="B23" s="18">
-        <f>IF(Tiers!$B$3="D. In-house media",IF(Costs!$B$22=1,Costs!$B$20,Costs!$B$19),Costs!$B$11)</f>
-        <v/>
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Yard sign and lockbox — cost</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="n">
+        <v>85</v>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>What the P&amp;L and unit economics use.</t>
+          <t>Sign amortized over about four listings, plus the box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Markup on add-ons</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Your 10%. See the note below before you count on this.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Fixed monthly — the brokerage exists whether or not anyone closes</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="n"/>
-      <c r="H25" s="20" t="n"/>
-      <c r="I25" s="20" t="n"/>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Share of listings buying flyers</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Brokerage E&amp;O policy</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="n">
-        <v>150</v>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>Firm policy. Agents carry their own on top.</t>
-        </is>
-      </c>
+          <t>Share of listings buying sign and lockbox</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>General liability</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="n">
-        <v>45</v>
-      </c>
-      <c r="C27" s="12" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Broker association and MLS dues</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n">
-        <v>85</v>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>Your own dues, annualized to a month.</t>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Add-on margin per listing</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>(B22*B25+B23*B26)*B24</f>
+        <v/>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Ten percent on about $130 of pass-through. It is a convenience, not a profit centre.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Website, hosting, domain, email</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C29" s="12" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Transaction management platform</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n">
-        <v>85</v>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>Base tier for a small firm.</t>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Active media cost per listing</t>
+        </is>
+      </c>
+      <c r="B29" s="18">
+        <f>IF(Tiers!$B$3="D. In-house media",IF(Costs!$B$20=1,Costs!$B$18,Costs!$B$17),Costs!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>What the P&amp;L and unit economics use.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>E-signature</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n">
-        <v>45</v>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>DocuSign Business Pro is about $45/user/month annually — needed for PowerForms.</t>
-        </is>
-      </c>
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Fixed monthly — the brokerage exists whether or not anyone closes</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="20" t="n"/>
+      <c r="E31" s="20" t="n"/>
+      <c r="F31" s="20" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="20" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Accounting and bookkeeping</t>
+          <t>Brokerage E&amp;O policy</t>
         </is>
       </c>
       <c r="B32" s="17" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Trust accounting is not a DIY job once agents are closing.</t>
+          <t>Firm policy. Agents carry their own on top.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Legal and compliance retainer</t>
+          <t>General liability</t>
         </is>
       </c>
       <c r="B33" s="17" t="n">
-        <v>125</v>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>Annual attorney review amortized.</t>
-        </is>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="C33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Phone system and call routing</t>
+          <t>Broker association and MLS dues</t>
         </is>
       </c>
       <c r="B34" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C34" s="12" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Your own dues, annualized to a month.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Banking, escrow account fees, software</t>
+          <t>Website, hosting, domain, email</t>
         </is>
       </c>
       <c r="B35" s="17" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Marketing and recruiting spend</t>
+          <t>Transaction management platform</t>
         </is>
       </c>
       <c r="B36" s="17" t="n">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Cards, cap hats, event table fees, boosted posts.</t>
+          <t>Base tier for a small firm.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Total fixed monthly</t>
-        </is>
-      </c>
-      <c r="B37" s="18">
-        <f>SUM(B26:B36)</f>
-        <v/>
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>E-signature</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>DocuSign Business Pro is about $45/user/month annually — needed for PowerForms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Accounting and bookkeeping</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="n">
+        <v>250</v>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Trust accounting is not a DIY job once agents are closing.</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Per agent, per month</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="20" t="n"/>
-      <c r="D39" s="20" t="n"/>
-      <c r="E39" s="20" t="n"/>
-      <c r="F39" s="20" t="n"/>
-      <c r="G39" s="20" t="n"/>
-      <c r="H39" s="20" t="n"/>
-      <c r="I39" s="20" t="n"/>
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Legal and compliance retainer</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="n">
+        <v>125</v>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Annual attorney review amortized.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>CRM seat</t>
+          <t>Phone system and call routing</t>
         </is>
       </c>
       <c r="B40" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>Follow Up Boss class tool. Only charged for tiers that include it.</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="C40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Email, storage, phone line</t>
+          <t>Banking, escrow account fees, software</t>
         </is>
       </c>
       <c r="B41" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>Charged for every agent.</t>
+        <v>40</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Marketing and recruiting spend</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Cards, cap hats, event table fees, boosted posts.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="inlineStr">
-        <is>
-          <t>Per transaction</t>
-        </is>
-      </c>
-      <c r="B43" s="20" t="n"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="E43" s="20" t="n"/>
-      <c r="F43" s="20" t="n"/>
-      <c r="G43" s="20" t="n"/>
-      <c r="H43" s="20" t="n"/>
-      <c r="I43" s="20" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
-        <is>
-          <t>Compliance review and file handling</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>Your time, costed. It is not free just because you do it.</t>
-        </is>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Total fixed monthly</t>
+        </is>
+      </c>
+      <c r="B43" s="18">
+        <f>SUM(B32:B42)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>Disbursement and banking</t>
-        </is>
-      </c>
-      <c r="B45" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="C45" s="12" t="inlineStr"/>
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Per agent, per month</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="n"/>
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="20" t="n"/>
+      <c r="E45" s="20" t="n"/>
+      <c r="F45" s="20" t="n"/>
+      <c r="G45" s="20" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
+          <t>CRM seat</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Follow Up Boss class tool. Only charged for tiers that include it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Email, storage, phone line</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Charged for every agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>Per transaction</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n"/>
+      <c r="C49" s="20" t="n"/>
+      <c r="D49" s="20" t="n"/>
+      <c r="E49" s="20" t="n"/>
+      <c r="F49" s="20" t="n"/>
+      <c r="G49" s="20" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Compliance review and file handling</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>Your time, costed. It is not free just because you do it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Disbursement and banking</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" s="12" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
           <t>Transaction coordination, when included</t>
         </is>
       </c>
-      <c r="B46" s="17" t="n">
+      <c r="B52" s="17" t="n">
         <v>325</v>
       </c>
-      <c r="C46" s="12" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>Outsourced TC per file. Only for tiers that include it.</t>
         </is>
@@ -2201,7 +2269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z29"/>
+  <dimension ref="A1:Z30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3112,99 +3180,99 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>B10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>B10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>C10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>C10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>D10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>D10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>E10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>E10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>F10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>F10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>G10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>G10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="H15" s="25">
-        <f>H10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>H10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="I15" s="25">
-        <f>I10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>I10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="J15" s="25">
-        <f>J10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>J10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="K15" s="25">
-        <f>K10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>K10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="L15" s="25">
-        <f>L10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>L10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="M15" s="25">
-        <f>M10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>M10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="N15" s="25">
-        <f>N10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>N10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="O15" s="25">
-        <f>O10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>O10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="P15" s="25">
-        <f>P10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>P10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Q15" s="25">
-        <f>Q10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>Q10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="R15" s="25">
-        <f>R10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>R10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="S15" s="25">
-        <f>S10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>S10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="T15" s="25">
-        <f>T10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>T10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="U15" s="25">
-        <f>U10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>U10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="V15" s="25">
-        <f>V10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>V10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="W15" s="25">
-        <f>W10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>W10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="X15" s="25">
-        <f>X10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>X10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Y15" s="25">
-        <f>Y10*MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>Y10*MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
       <c r="Z15" s="18">
@@ -3213,105 +3281,105 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Total revenue</t>
-        </is>
-      </c>
-      <c r="B16" s="18">
-        <f>SUM(B13:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="18">
-        <f>SUM(C13:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="18">
-        <f>SUM(D13:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="18">
-        <f>SUM(E13:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="18">
-        <f>SUM(F13:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="18">
-        <f>SUM(G13:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="18">
-        <f>SUM(H13:H15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="18">
-        <f>SUM(I13:I15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="18">
-        <f>SUM(J13:J15)</f>
-        <v/>
-      </c>
-      <c r="K16" s="18">
-        <f>SUM(K13:K15)</f>
-        <v/>
-      </c>
-      <c r="L16" s="18">
-        <f>SUM(L13:L15)</f>
-        <v/>
-      </c>
-      <c r="M16" s="18">
-        <f>SUM(M13:M15)</f>
-        <v/>
-      </c>
-      <c r="N16" s="18">
-        <f>SUM(N13:N15)</f>
-        <v/>
-      </c>
-      <c r="O16" s="18">
-        <f>SUM(O13:O15)</f>
-        <v/>
-      </c>
-      <c r="P16" s="18">
-        <f>SUM(P13:P15)</f>
-        <v/>
-      </c>
-      <c r="Q16" s="18">
-        <f>SUM(Q13:Q15)</f>
-        <v/>
-      </c>
-      <c r="R16" s="18">
-        <f>SUM(R13:R15)</f>
-        <v/>
-      </c>
-      <c r="S16" s="18">
-        <f>SUM(S13:S15)</f>
-        <v/>
-      </c>
-      <c r="T16" s="18">
-        <f>SUM(T13:T15)</f>
-        <v/>
-      </c>
-      <c r="U16" s="18">
-        <f>SUM(U13:U15)</f>
-        <v/>
-      </c>
-      <c r="V16" s="18">
-        <f>SUM(V13:V15)</f>
-        <v/>
-      </c>
-      <c r="W16" s="18">
-        <f>SUM(W13:W15)</f>
-        <v/>
-      </c>
-      <c r="X16" s="18">
-        <f>SUM(X13:X15)</f>
-        <v/>
-      </c>
-      <c r="Y16" s="18">
-        <f>SUM(Y13:Y15)</f>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Add-on margin (flyers, sign, lockbox)</t>
+        </is>
+      </c>
+      <c r="B16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",B9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="C16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",C9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",D9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",E9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",F9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",G9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="H16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",H9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="I16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",I9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="J16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",J9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="K16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",K9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="L16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",L9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="M16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",M9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="N16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",N9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="O16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",O9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="P16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",P9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",Q9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="R16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",R9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="S16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",S9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="T16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",T9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="U16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",U9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="V16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",V9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="W16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",W9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="X16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",X9*Costs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="Y16" s="25">
+        <f>IF(Tiers!$B$3="D. In-house media",Y9*Costs!$B$27,0)</f>
         <v/>
       </c>
       <c r="Z16" s="18">
@@ -3319,231 +3387,231 @@
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B17" s="18">
+        <f>SUM(B13:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="18">
+        <f>SUM(C13:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="18">
+        <f>SUM(D13:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>SUM(E13:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="18">
+        <f>SUM(F13:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="18">
+        <f>SUM(G13:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="18">
+        <f>SUM(H13:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="18">
+        <f>SUM(I13:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="18">
+        <f>SUM(J13:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="18">
+        <f>SUM(K13:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>SUM(L13:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="18">
+        <f>SUM(M13:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="18">
+        <f>SUM(N13:N16)</f>
+        <v/>
+      </c>
+      <c r="O17" s="18">
+        <f>SUM(O13:O16)</f>
+        <v/>
+      </c>
+      <c r="P17" s="18">
+        <f>SUM(P13:P16)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="18">
+        <f>SUM(Q13:Q16)</f>
+        <v/>
+      </c>
+      <c r="R17" s="18">
+        <f>SUM(R13:R16)</f>
+        <v/>
+      </c>
+      <c r="S17" s="18">
+        <f>SUM(S13:S16)</f>
+        <v/>
+      </c>
+      <c r="T17" s="18">
+        <f>SUM(T13:T16)</f>
+        <v/>
+      </c>
+      <c r="U17" s="18">
+        <f>SUM(U13:U16)</f>
+        <v/>
+      </c>
+      <c r="V17" s="18">
+        <f>SUM(V13:V16)</f>
+        <v/>
+      </c>
+      <c r="W17" s="18">
+        <f>SUM(W13:W16)</f>
+        <v/>
+      </c>
+      <c r="X17" s="18">
+        <f>SUM(X13:X16)</f>
+        <v/>
+      </c>
+      <c r="Y17" s="18">
+        <f>SUM(Y13:Y16)</f>
+        <v/>
+      </c>
+      <c r="Z17" s="18">
+        <f>SUM(B17:Y17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Cost of service</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="20" t="n"/>
-      <c r="I18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Listings above your shooting capacity</t>
-        </is>
-      </c>
-      <c r="B19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,B10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="C19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,C10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="D19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,D10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="E19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,E10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="F19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,F10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="G19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,G10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="H19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,H10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="I19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,I10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="J19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,J10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="K19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,K10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="L19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,L10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="M19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,M10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="N19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,N10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="O19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,O10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="P19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,P10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="Q19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Q10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="R19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,R10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="S19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,S10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="T19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,T10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="U19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,U10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="V19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,V10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="W19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,W10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="X19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,X10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="Y19" s="24">
-        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Y10-Costs!$B$21),0)</f>
-        <v/>
-      </c>
-      <c r="Z19" s="14">
-        <f>SUM(B19:Y19)</f>
-        <v/>
-      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Media cost</t>
-        </is>
-      </c>
-      <c r="B20" s="25">
-        <f>MIN(B10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,B10))*Costs!$B$23+B19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="C20" s="25">
-        <f>MIN(C10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,C10))*Costs!$B$23+C19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="D20" s="25">
-        <f>MIN(D10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,D10))*Costs!$B$23+D19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="E20" s="25">
-        <f>MIN(E10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,E10))*Costs!$B$23+E19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="F20" s="25">
-        <f>MIN(F10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,F10))*Costs!$B$23+F19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="G20" s="25">
-        <f>MIN(G10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,G10))*Costs!$B$23+G19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="H20" s="25">
-        <f>MIN(H10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,H10))*Costs!$B$23+H19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="I20" s="25">
-        <f>MIN(I10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,I10))*Costs!$B$23+I19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="J20" s="25">
-        <f>MIN(J10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,J10))*Costs!$B$23+J19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="K20" s="25">
-        <f>MIN(K10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,K10))*Costs!$B$23+K19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="L20" s="25">
-        <f>MIN(L10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,L10))*Costs!$B$23+L19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="M20" s="25">
-        <f>MIN(M10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,M10))*Costs!$B$23+M19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="N20" s="25">
-        <f>MIN(N10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,N10))*Costs!$B$23+N19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="O20" s="25">
-        <f>MIN(O10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,O10))*Costs!$B$23+O19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="P20" s="25">
-        <f>MIN(P10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,P10))*Costs!$B$23+P19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Q20" s="25">
-        <f>MIN(Q10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,Q10))*Costs!$B$23+Q19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="R20" s="25">
-        <f>MIN(R10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,R10))*Costs!$B$23+R19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="S20" s="25">
-        <f>MIN(S10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,S10))*Costs!$B$23+S19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="T20" s="25">
-        <f>MIN(T10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,T10))*Costs!$B$23+T19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="U20" s="25">
-        <f>MIN(U10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,U10))*Costs!$B$23+U19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="V20" s="25">
-        <f>MIN(V10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,V10))*Costs!$B$23+V19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="W20" s="25">
-        <f>MIN(W10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,W10))*Costs!$B$23+W19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="X20" s="25">
-        <f>MIN(X10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,X10))*Costs!$B$23+X19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Y20" s="25">
-        <f>MIN(Y10,IF(Tiers!$B$3="D. In-house media",Costs!$B$21,Y10))*Costs!$B$23+Y19*Costs!$B$11</f>
-        <v/>
-      </c>
-      <c r="Z20" s="18">
+          <t>Listings above your shooting capacity</t>
+        </is>
+      </c>
+      <c r="B20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,B10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="C20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,C10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,D10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="E20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,E10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,F10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,G10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="H20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,H10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="I20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,I10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="J20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,J10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="K20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,K10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="L20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,L10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="M20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,M10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="N20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,N10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="O20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,O10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="P20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,P10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Q10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="R20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,R10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="S20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,S10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="T20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,T10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="U20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,U10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="V20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,V10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="W20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,W10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="X20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,X10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="Y20" s="24">
+        <f>IF(Tiers!$B$3="D. In-house media",MAX(0,Y10-Costs!$B$19),0)</f>
+        <v/>
+      </c>
+      <c r="Z20" s="14">
         <f>SUM(B20:Y20)</f>
         <v/>
       </c>
@@ -3551,103 +3619,103 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Per-transaction cost</t>
+          <t>Media cost</t>
         </is>
       </c>
       <c r="B21" s="25">
-        <f>B8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(B10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,B10))*Costs!$B$29+B20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>C8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(C10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,C10))*Costs!$B$29+C20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>D8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(D10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,D10))*Costs!$B$29+D20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="E21" s="25">
-        <f>E8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(E10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,E10))*Costs!$B$29+E20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="F21" s="25">
-        <f>F8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(F10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,F10))*Costs!$B$29+F20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="G21" s="25">
-        <f>G8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(G10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,G10))*Costs!$B$29+G20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="H21" s="25">
-        <f>H8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(H10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,H10))*Costs!$B$29+H20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="I21" s="25">
-        <f>I8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(I10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,I10))*Costs!$B$29+I20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="J21" s="25">
-        <f>J8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(J10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,J10))*Costs!$B$29+J20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="K21" s="25">
-        <f>K8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(K10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,K10))*Costs!$B$29+K20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="L21" s="25">
-        <f>L8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(L10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,L10))*Costs!$B$29+L20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="M21" s="25">
-        <f>M8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(M10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,M10))*Costs!$B$29+M20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="N21" s="25">
-        <f>N8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(N10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,N10))*Costs!$B$29+N20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="O21" s="25">
-        <f>O8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(O10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,O10))*Costs!$B$29+O20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="P21" s="25">
-        <f>P8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(P10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,P10))*Costs!$B$29+P20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Q21" s="25">
-        <f>Q8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(Q10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,Q10))*Costs!$B$29+Q20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="R21" s="25">
-        <f>R8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(R10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,R10))*Costs!$B$29+R20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="S21" s="25">
-        <f>S8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(S10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,S10))*Costs!$B$29+S20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="T21" s="25">
-        <f>T8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(T10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,T10))*Costs!$B$29+T20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="U21" s="25">
-        <f>U8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(U10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,U10))*Costs!$B$29+U20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="V21" s="25">
-        <f>V8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(V10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,V10))*Costs!$B$29+V20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="W21" s="25">
-        <f>W8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(W10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,W10))*Costs!$B$29+W20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="X21" s="25">
-        <f>X8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(X10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,X10))*Costs!$B$29+X20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Y21" s="25">
-        <f>Y8*((Costs!$B$44+Costs!$B$45)+Tiers!$B$25*Costs!$B$46)</f>
+        <f>MIN(Y10,IF(Tiers!$B$3="D. In-house media",Costs!$B$19,Y10))*Costs!$B$29+Y20*Costs!$B$11</f>
         <v/>
       </c>
       <c r="Z21" s="18">
@@ -3658,103 +3726,103 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Per-agent cost</t>
+          <t>Per-transaction cost</t>
         </is>
       </c>
       <c r="B22" s="25">
-        <f>B7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>B8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>C7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>C8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="D22" s="25">
-        <f>D7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>D8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="E22" s="25">
-        <f>E7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>E8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="F22" s="25">
-        <f>F7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>F8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="G22" s="25">
-        <f>G7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>G8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="H22" s="25">
-        <f>H7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>H8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="I22" s="25">
-        <f>I7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>I8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="J22" s="25">
-        <f>J7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>J8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="K22" s="25">
-        <f>K7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>K8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="L22" s="25">
-        <f>L7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>L8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="M22" s="25">
-        <f>M7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>M8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="N22" s="25">
-        <f>N7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>N8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="O22" s="25">
-        <f>O7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>O8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="P22" s="25">
-        <f>P7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>P8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="Q22" s="25">
-        <f>Q7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>Q8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="R22" s="25">
-        <f>R7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>R8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="S22" s="25">
-        <f>S7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>S8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="T22" s="25">
-        <f>T7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>T8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="U22" s="25">
-        <f>U7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>U8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="V22" s="25">
-        <f>V7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>V8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="W22" s="25">
-        <f>W7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>W8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="X22" s="25">
-        <f>X7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>X8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="Y22" s="25">
-        <f>Y7*(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>Y8*((Costs!$B$50+Costs!$B$51)+Tiers!$B$25*Costs!$B$52)</f>
         <v/>
       </c>
       <c r="Z22" s="18">
@@ -3765,103 +3833,103 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Fixed overhead</t>
+          <t>Per-agent cost</t>
         </is>
       </c>
       <c r="B23" s="25">
-        <f>Costs!$B$37</f>
+        <f>B7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>Costs!$B$37</f>
+        <f>C7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="D23" s="25">
-        <f>Costs!$B$37</f>
+        <f>D7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="E23" s="25">
-        <f>Costs!$B$37</f>
+        <f>E7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="F23" s="25">
-        <f>Costs!$B$37</f>
+        <f>F7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="G23" s="25">
-        <f>Costs!$B$37</f>
+        <f>G7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="H23" s="25">
-        <f>Costs!$B$37</f>
+        <f>H7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="I23" s="25">
-        <f>Costs!$B$37</f>
+        <f>I7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="J23" s="25">
-        <f>Costs!$B$37</f>
+        <f>J7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="K23" s="25">
-        <f>Costs!$B$37</f>
+        <f>K7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="L23" s="25">
-        <f>Costs!$B$37</f>
+        <f>L7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="M23" s="25">
-        <f>Costs!$B$37</f>
+        <f>M7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="N23" s="25">
-        <f>Costs!$B$37</f>
+        <f>N7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="O23" s="25">
-        <f>Costs!$B$37</f>
+        <f>O7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="P23" s="25">
-        <f>Costs!$B$37</f>
+        <f>P7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Q23" s="25">
-        <f>Costs!$B$37</f>
+        <f>Q7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="R23" s="25">
-        <f>Costs!$B$37</f>
+        <f>R7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="S23" s="25">
-        <f>Costs!$B$37</f>
+        <f>S7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="T23" s="25">
-        <f>Costs!$B$37</f>
+        <f>T7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="U23" s="25">
-        <f>Costs!$B$37</f>
+        <f>U7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="V23" s="25">
-        <f>Costs!$B$37</f>
+        <f>V7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="W23" s="25">
-        <f>Costs!$B$37</f>
+        <f>W7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="X23" s="25">
-        <f>Costs!$B$37</f>
+        <f>X7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Y23" s="25">
-        <f>Costs!$B$37</f>
+        <f>Y7*(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
         <v/>
       </c>
       <c r="Z23" s="18">
@@ -3872,103 +3940,103 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Managing agent compensation</t>
+          <t>Fixed overhead</t>
         </is>
       </c>
       <c r="B24" s="25">
-        <f>'Managing Agent'!B$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="C24" s="25">
-        <f>'Managing Agent'!C$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="D24" s="25">
-        <f>'Managing Agent'!D$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="E24" s="25">
-        <f>'Managing Agent'!E$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="F24" s="25">
-        <f>'Managing Agent'!F$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="G24" s="25">
-        <f>'Managing Agent'!G$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="H24" s="25">
-        <f>'Managing Agent'!H$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="I24" s="25">
-        <f>'Managing Agent'!I$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="J24" s="25">
-        <f>'Managing Agent'!J$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="K24" s="25">
-        <f>'Managing Agent'!K$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="L24" s="25">
-        <f>'Managing Agent'!L$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="M24" s="25">
-        <f>'Managing Agent'!M$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="N24" s="25">
-        <f>'Managing Agent'!N$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="O24" s="25">
-        <f>'Managing Agent'!O$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="P24" s="25">
-        <f>'Managing Agent'!P$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="Q24" s="25">
-        <f>'Managing Agent'!Q$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="R24" s="25">
-        <f>'Managing Agent'!R$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="S24" s="25">
-        <f>'Managing Agent'!S$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="T24" s="25">
-        <f>'Managing Agent'!T$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="U24" s="25">
-        <f>'Managing Agent'!U$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="V24" s="25">
-        <f>'Managing Agent'!V$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="W24" s="25">
-        <f>'Managing Agent'!W$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="X24" s="25">
-        <f>'Managing Agent'!X$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="Y24" s="25">
-        <f>'Managing Agent'!Y$30</f>
+        <f>Costs!$B$43</f>
         <v/>
       </c>
       <c r="Z24" s="18">
@@ -3977,105 +4045,105 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Total cost</t>
-        </is>
-      </c>
-      <c r="B25" s="18">
-        <f>SUM(B20:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="18">
-        <f>SUM(C20:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="18">
-        <f>SUM(D20:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="18">
-        <f>SUM(E20:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="18">
-        <f>SUM(F20:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="18">
-        <f>SUM(G20:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="18">
-        <f>SUM(H20:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="18">
-        <f>SUM(I20:I24)</f>
-        <v/>
-      </c>
-      <c r="J25" s="18">
-        <f>SUM(J20:J24)</f>
-        <v/>
-      </c>
-      <c r="K25" s="18">
-        <f>SUM(K20:K24)</f>
-        <v/>
-      </c>
-      <c r="L25" s="18">
-        <f>SUM(L20:L24)</f>
-        <v/>
-      </c>
-      <c r="M25" s="18">
-        <f>SUM(M20:M24)</f>
-        <v/>
-      </c>
-      <c r="N25" s="18">
-        <f>SUM(N20:N24)</f>
-        <v/>
-      </c>
-      <c r="O25" s="18">
-        <f>SUM(O20:O24)</f>
-        <v/>
-      </c>
-      <c r="P25" s="18">
-        <f>SUM(P20:P24)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="18">
-        <f>SUM(Q20:Q24)</f>
-        <v/>
-      </c>
-      <c r="R25" s="18">
-        <f>SUM(R20:R24)</f>
-        <v/>
-      </c>
-      <c r="S25" s="18">
-        <f>SUM(S20:S24)</f>
-        <v/>
-      </c>
-      <c r="T25" s="18">
-        <f>SUM(T20:T24)</f>
-        <v/>
-      </c>
-      <c r="U25" s="18">
-        <f>SUM(U20:U24)</f>
-        <v/>
-      </c>
-      <c r="V25" s="18">
-        <f>SUM(V20:V24)</f>
-        <v/>
-      </c>
-      <c r="W25" s="18">
-        <f>SUM(W20:W24)</f>
-        <v/>
-      </c>
-      <c r="X25" s="18">
-        <f>SUM(X20:X24)</f>
-        <v/>
-      </c>
-      <c r="Y25" s="18">
-        <f>SUM(Y20:Y24)</f>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Managing agent compensation</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>'Managing Agent'!B$30</f>
+        <v/>
+      </c>
+      <c r="C25" s="25">
+        <f>'Managing Agent'!C$30</f>
+        <v/>
+      </c>
+      <c r="D25" s="25">
+        <f>'Managing Agent'!D$30</f>
+        <v/>
+      </c>
+      <c r="E25" s="25">
+        <f>'Managing Agent'!E$30</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>'Managing Agent'!F$30</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>'Managing Agent'!G$30</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>'Managing Agent'!H$30</f>
+        <v/>
+      </c>
+      <c r="I25" s="25">
+        <f>'Managing Agent'!I$30</f>
+        <v/>
+      </c>
+      <c r="J25" s="25">
+        <f>'Managing Agent'!J$30</f>
+        <v/>
+      </c>
+      <c r="K25" s="25">
+        <f>'Managing Agent'!K$30</f>
+        <v/>
+      </c>
+      <c r="L25" s="25">
+        <f>'Managing Agent'!L$30</f>
+        <v/>
+      </c>
+      <c r="M25" s="25">
+        <f>'Managing Agent'!M$30</f>
+        <v/>
+      </c>
+      <c r="N25" s="25">
+        <f>'Managing Agent'!N$30</f>
+        <v/>
+      </c>
+      <c r="O25" s="25">
+        <f>'Managing Agent'!O$30</f>
+        <v/>
+      </c>
+      <c r="P25" s="25">
+        <f>'Managing Agent'!P$30</f>
+        <v/>
+      </c>
+      <c r="Q25" s="25">
+        <f>'Managing Agent'!Q$30</f>
+        <v/>
+      </c>
+      <c r="R25" s="25">
+        <f>'Managing Agent'!R$30</f>
+        <v/>
+      </c>
+      <c r="S25" s="25">
+        <f>'Managing Agent'!S$30</f>
+        <v/>
+      </c>
+      <c r="T25" s="25">
+        <f>'Managing Agent'!T$30</f>
+        <v/>
+      </c>
+      <c r="U25" s="25">
+        <f>'Managing Agent'!U$30</f>
+        <v/>
+      </c>
+      <c r="V25" s="25">
+        <f>'Managing Agent'!V$30</f>
+        <v/>
+      </c>
+      <c r="W25" s="25">
+        <f>'Managing Agent'!W$30</f>
+        <v/>
+      </c>
+      <c r="X25" s="25">
+        <f>'Managing Agent'!X$30</f>
+        <v/>
+      </c>
+      <c r="Y25" s="25">
+        <f>'Managing Agent'!Y$30</f>
         <v/>
       </c>
       <c r="Z25" s="18">
@@ -4083,324 +4151,431 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B27" s="18">
-        <f>B16-B25</f>
-        <v/>
-      </c>
-      <c r="C27" s="18">
-        <f>C16-C25</f>
-        <v/>
-      </c>
-      <c r="D27" s="18">
-        <f>D16-D25</f>
-        <v/>
-      </c>
-      <c r="E27" s="18">
-        <f>E16-E25</f>
-        <v/>
-      </c>
-      <c r="F27" s="18">
-        <f>F16-F25</f>
-        <v/>
-      </c>
-      <c r="G27" s="18">
-        <f>G16-G25</f>
-        <v/>
-      </c>
-      <c r="H27" s="18">
-        <f>H16-H25</f>
-        <v/>
-      </c>
-      <c r="I27" s="18">
-        <f>I16-I25</f>
-        <v/>
-      </c>
-      <c r="J27" s="18">
-        <f>J16-J25</f>
-        <v/>
-      </c>
-      <c r="K27" s="18">
-        <f>K16-K25</f>
-        <v/>
-      </c>
-      <c r="L27" s="18">
-        <f>L16-L25</f>
-        <v/>
-      </c>
-      <c r="M27" s="18">
-        <f>M16-M25</f>
-        <v/>
-      </c>
-      <c r="N27" s="18">
-        <f>N16-N25</f>
-        <v/>
-      </c>
-      <c r="O27" s="18">
-        <f>O16-O25</f>
-        <v/>
-      </c>
-      <c r="P27" s="18">
-        <f>P16-P25</f>
-        <v/>
-      </c>
-      <c r="Q27" s="18">
-        <f>Q16-Q25</f>
-        <v/>
-      </c>
-      <c r="R27" s="18">
-        <f>R16-R25</f>
-        <v/>
-      </c>
-      <c r="S27" s="18">
-        <f>S16-S25</f>
-        <v/>
-      </c>
-      <c r="T27" s="18">
-        <f>T16-T25</f>
-        <v/>
-      </c>
-      <c r="U27" s="18">
-        <f>U16-U25</f>
-        <v/>
-      </c>
-      <c r="V27" s="18">
-        <f>V16-V25</f>
-        <v/>
-      </c>
-      <c r="W27" s="18">
-        <f>W16-W25</f>
-        <v/>
-      </c>
-      <c r="X27" s="18">
-        <f>X16-X25</f>
-        <v/>
-      </c>
-      <c r="Y27" s="18">
-        <f>Y16-Y25</f>
-        <v/>
-      </c>
-      <c r="Z27" s="18">
-        <f>SUM(B27:Y27)</f>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Total cost</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>SUM(B21:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="18">
+        <f>SUM(C21:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="18">
+        <f>SUM(D21:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="18">
+        <f>SUM(E21:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="18">
+        <f>SUM(F21:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="18">
+        <f>SUM(G21:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="18">
+        <f>SUM(H21:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="18">
+        <f>SUM(I21:I25)</f>
+        <v/>
+      </c>
+      <c r="J26" s="18">
+        <f>SUM(J21:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="18">
+        <f>SUM(K21:K25)</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>SUM(L21:L25)</f>
+        <v/>
+      </c>
+      <c r="M26" s="18">
+        <f>SUM(M21:M25)</f>
+        <v/>
+      </c>
+      <c r="N26" s="18">
+        <f>SUM(N21:N25)</f>
+        <v/>
+      </c>
+      <c r="O26" s="18">
+        <f>SUM(O21:O25)</f>
+        <v/>
+      </c>
+      <c r="P26" s="18">
+        <f>SUM(P21:P25)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="18">
+        <f>SUM(Q21:Q25)</f>
+        <v/>
+      </c>
+      <c r="R26" s="18">
+        <f>SUM(R21:R25)</f>
+        <v/>
+      </c>
+      <c r="S26" s="18">
+        <f>SUM(S21:S25)</f>
+        <v/>
+      </c>
+      <c r="T26" s="18">
+        <f>SUM(T21:T25)</f>
+        <v/>
+      </c>
+      <c r="U26" s="18">
+        <f>SUM(U21:U25)</f>
+        <v/>
+      </c>
+      <c r="V26" s="18">
+        <f>SUM(V21:V25)</f>
+        <v/>
+      </c>
+      <c r="W26" s="18">
+        <f>SUM(W21:W25)</f>
+        <v/>
+      </c>
+      <c r="X26" s="18">
+        <f>SUM(X21:X25)</f>
+        <v/>
+      </c>
+      <c r="Y26" s="18">
+        <f>SUM(Y21:Y25)</f>
+        <v/>
+      </c>
+      <c r="Z26" s="18">
+        <f>SUM(B26:Y26)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B28" s="18">
+        <f>B17-B26</f>
+        <v/>
+      </c>
+      <c r="C28" s="18">
+        <f>C17-C26</f>
+        <v/>
+      </c>
+      <c r="D28" s="18">
+        <f>D17-D26</f>
+        <v/>
+      </c>
+      <c r="E28" s="18">
+        <f>E17-E26</f>
+        <v/>
+      </c>
+      <c r="F28" s="18">
+        <f>F17-F26</f>
+        <v/>
+      </c>
+      <c r="G28" s="18">
+        <f>G17-G26</f>
+        <v/>
+      </c>
+      <c r="H28" s="18">
+        <f>H17-H26</f>
+        <v/>
+      </c>
+      <c r="I28" s="18">
+        <f>I17-I26</f>
+        <v/>
+      </c>
+      <c r="J28" s="18">
+        <f>J17-J26</f>
+        <v/>
+      </c>
+      <c r="K28" s="18">
+        <f>K17-K26</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>L17-L26</f>
+        <v/>
+      </c>
+      <c r="M28" s="18">
+        <f>M17-M26</f>
+        <v/>
+      </c>
+      <c r="N28" s="18">
+        <f>N17-N26</f>
+        <v/>
+      </c>
+      <c r="O28" s="18">
+        <f>O17-O26</f>
+        <v/>
+      </c>
+      <c r="P28" s="18">
+        <f>P17-P26</f>
+        <v/>
+      </c>
+      <c r="Q28" s="18">
+        <f>Q17-Q26</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>R17-R26</f>
+        <v/>
+      </c>
+      <c r="S28" s="18">
+        <f>S17-S26</f>
+        <v/>
+      </c>
+      <c r="T28" s="18">
+        <f>T17-T26</f>
+        <v/>
+      </c>
+      <c r="U28" s="18">
+        <f>U17-U26</f>
+        <v/>
+      </c>
+      <c r="V28" s="18">
+        <f>V17-V26</f>
+        <v/>
+      </c>
+      <c r="W28" s="18">
+        <f>W17-W26</f>
+        <v/>
+      </c>
+      <c r="X28" s="18">
+        <f>X17-X26</f>
+        <v/>
+      </c>
+      <c r="Y28" s="18">
+        <f>Y17-Y26</f>
+        <v/>
+      </c>
+      <c r="Z28" s="18">
+        <f>SUM(B28:Y28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>Cumulative EBITDA</t>
         </is>
       </c>
-      <c r="B28" s="18">
-        <f>B27</f>
-        <v/>
-      </c>
-      <c r="C28" s="18">
-        <f>B28+C27</f>
-        <v/>
-      </c>
-      <c r="D28" s="18">
-        <f>C28+D27</f>
-        <v/>
-      </c>
-      <c r="E28" s="18">
-        <f>D28+E27</f>
-        <v/>
-      </c>
-      <c r="F28" s="18">
-        <f>E28+F27</f>
-        <v/>
-      </c>
-      <c r="G28" s="18">
-        <f>F28+G27</f>
-        <v/>
-      </c>
-      <c r="H28" s="18">
-        <f>G28+H27</f>
-        <v/>
-      </c>
-      <c r="I28" s="18">
-        <f>H28+I27</f>
-        <v/>
-      </c>
-      <c r="J28" s="18">
-        <f>I28+J27</f>
-        <v/>
-      </c>
-      <c r="K28" s="18">
-        <f>J28+K27</f>
-        <v/>
-      </c>
-      <c r="L28" s="18">
-        <f>K28+L27</f>
-        <v/>
-      </c>
-      <c r="M28" s="18">
-        <f>L28+M27</f>
-        <v/>
-      </c>
-      <c r="N28" s="18">
-        <f>M28+N27</f>
-        <v/>
-      </c>
-      <c r="O28" s="18">
-        <f>N28+O27</f>
-        <v/>
-      </c>
-      <c r="P28" s="18">
-        <f>O28+P27</f>
-        <v/>
-      </c>
-      <c r="Q28" s="18">
-        <f>P28+Q27</f>
-        <v/>
-      </c>
-      <c r="R28" s="18">
-        <f>Q28+R27</f>
-        <v/>
-      </c>
-      <c r="S28" s="18">
-        <f>R28+S27</f>
-        <v/>
-      </c>
-      <c r="T28" s="18">
-        <f>S28+T27</f>
-        <v/>
-      </c>
-      <c r="U28" s="18">
-        <f>T28+U27</f>
-        <v/>
-      </c>
-      <c r="V28" s="18">
-        <f>U28+V27</f>
-        <v/>
-      </c>
-      <c r="W28" s="18">
-        <f>V28+W27</f>
-        <v/>
-      </c>
-      <c r="X28" s="18">
-        <f>W28+X27</f>
-        <v/>
-      </c>
-      <c r="Y28" s="18">
-        <f>X28+Y27</f>
-        <v/>
-      </c>
-      <c r="Z28" s="18">
-        <f>Y28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="B29" s="18">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="18">
+        <f>B29+C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="18">
+        <f>C29+D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="18">
+        <f>D29+E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="18">
+        <f>E29+F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="18">
+        <f>F29+G28</f>
+        <v/>
+      </c>
+      <c r="H29" s="18">
+        <f>G29+H28</f>
+        <v/>
+      </c>
+      <c r="I29" s="18">
+        <f>H29+I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="18">
+        <f>I29+J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="18">
+        <f>J29+K28</f>
+        <v/>
+      </c>
+      <c r="L29" s="18">
+        <f>K29+L28</f>
+        <v/>
+      </c>
+      <c r="M29" s="18">
+        <f>L29+M28</f>
+        <v/>
+      </c>
+      <c r="N29" s="18">
+        <f>M29+N28</f>
+        <v/>
+      </c>
+      <c r="O29" s="18">
+        <f>N29+O28</f>
+        <v/>
+      </c>
+      <c r="P29" s="18">
+        <f>O29+P28</f>
+        <v/>
+      </c>
+      <c r="Q29" s="18">
+        <f>P29+Q28</f>
+        <v/>
+      </c>
+      <c r="R29" s="18">
+        <f>Q29+R28</f>
+        <v/>
+      </c>
+      <c r="S29" s="18">
+        <f>R29+S28</f>
+        <v/>
+      </c>
+      <c r="T29" s="18">
+        <f>S29+T28</f>
+        <v/>
+      </c>
+      <c r="U29" s="18">
+        <f>T29+U28</f>
+        <v/>
+      </c>
+      <c r="V29" s="18">
+        <f>U29+V28</f>
+        <v/>
+      </c>
+      <c r="W29" s="18">
+        <f>V29+W28</f>
+        <v/>
+      </c>
+      <c r="X29" s="18">
+        <f>W29+X28</f>
+        <v/>
+      </c>
+      <c r="Y29" s="18">
+        <f>X29+Y28</f>
+        <v/>
+      </c>
+      <c r="Z29" s="18">
+        <f>Y29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>EBITDA margin</t>
         </is>
       </c>
-      <c r="B29" s="26">
-        <f>IFERROR(B27/B16,0)</f>
-        <v/>
-      </c>
-      <c r="C29" s="26">
-        <f>IFERROR(C27/C16,0)</f>
-        <v/>
-      </c>
-      <c r="D29" s="26">
-        <f>IFERROR(D27/D16,0)</f>
-        <v/>
-      </c>
-      <c r="E29" s="26">
-        <f>IFERROR(E27/E16,0)</f>
-        <v/>
-      </c>
-      <c r="F29" s="26">
-        <f>IFERROR(F27/F16,0)</f>
-        <v/>
-      </c>
-      <c r="G29" s="26">
-        <f>IFERROR(G27/G16,0)</f>
-        <v/>
-      </c>
-      <c r="H29" s="26">
-        <f>IFERROR(H27/H16,0)</f>
-        <v/>
-      </c>
-      <c r="I29" s="26">
-        <f>IFERROR(I27/I16,0)</f>
-        <v/>
-      </c>
-      <c r="J29" s="26">
-        <f>IFERROR(J27/J16,0)</f>
-        <v/>
-      </c>
-      <c r="K29" s="26">
-        <f>IFERROR(K27/K16,0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="26">
-        <f>IFERROR(L27/L16,0)</f>
-        <v/>
-      </c>
-      <c r="M29" s="26">
-        <f>IFERROR(M27/M16,0)</f>
-        <v/>
-      </c>
-      <c r="N29" s="26">
-        <f>IFERROR(N27/N16,0)</f>
-        <v/>
-      </c>
-      <c r="O29" s="26">
-        <f>IFERROR(O27/O16,0)</f>
-        <v/>
-      </c>
-      <c r="P29" s="26">
-        <f>IFERROR(P27/P16,0)</f>
-        <v/>
-      </c>
-      <c r="Q29" s="26">
-        <f>IFERROR(Q27/Q16,0)</f>
-        <v/>
-      </c>
-      <c r="R29" s="26">
-        <f>IFERROR(R27/R16,0)</f>
-        <v/>
-      </c>
-      <c r="S29" s="26">
-        <f>IFERROR(S27/S16,0)</f>
-        <v/>
-      </c>
-      <c r="T29" s="26">
-        <f>IFERROR(T27/T16,0)</f>
-        <v/>
-      </c>
-      <c r="U29" s="26">
-        <f>IFERROR(U27/U16,0)</f>
-        <v/>
-      </c>
-      <c r="V29" s="26">
-        <f>IFERROR(V27/V16,0)</f>
-        <v/>
-      </c>
-      <c r="W29" s="26">
-        <f>IFERROR(W27/W16,0)</f>
-        <v/>
-      </c>
-      <c r="X29" s="26">
-        <f>IFERROR(X27/X16,0)</f>
-        <v/>
-      </c>
-      <c r="Y29" s="26">
-        <f>IFERROR(Y27/Y16,0)</f>
-        <v/>
-      </c>
-      <c r="Z29" s="16">
-        <f>IFERROR(Z27/Z16,0)</f>
+      <c r="B30" s="26">
+        <f>IFERROR(B28/B17,0)</f>
+        <v/>
+      </c>
+      <c r="C30" s="26">
+        <f>IFERROR(C28/C17,0)</f>
+        <v/>
+      </c>
+      <c r="D30" s="26">
+        <f>IFERROR(D28/D17,0)</f>
+        <v/>
+      </c>
+      <c r="E30" s="26">
+        <f>IFERROR(E28/E17,0)</f>
+        <v/>
+      </c>
+      <c r="F30" s="26">
+        <f>IFERROR(F28/F17,0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="26">
+        <f>IFERROR(G28/G17,0)</f>
+        <v/>
+      </c>
+      <c r="H30" s="26">
+        <f>IFERROR(H28/H17,0)</f>
+        <v/>
+      </c>
+      <c r="I30" s="26">
+        <f>IFERROR(I28/I17,0)</f>
+        <v/>
+      </c>
+      <c r="J30" s="26">
+        <f>IFERROR(J28/J17,0)</f>
+        <v/>
+      </c>
+      <c r="K30" s="26">
+        <f>IFERROR(K28/K17,0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="26">
+        <f>IFERROR(L28/L17,0)</f>
+        <v/>
+      </c>
+      <c r="M30" s="26">
+        <f>IFERROR(M28/M17,0)</f>
+        <v/>
+      </c>
+      <c r="N30" s="26">
+        <f>IFERROR(N28/N17,0)</f>
+        <v/>
+      </c>
+      <c r="O30" s="26">
+        <f>IFERROR(O28/O17,0)</f>
+        <v/>
+      </c>
+      <c r="P30" s="26">
+        <f>IFERROR(P28/P17,0)</f>
+        <v/>
+      </c>
+      <c r="Q30" s="26">
+        <f>IFERROR(Q28/Q17,0)</f>
+        <v/>
+      </c>
+      <c r="R30" s="26">
+        <f>IFERROR(R28/R17,0)</f>
+        <v/>
+      </c>
+      <c r="S30" s="26">
+        <f>IFERROR(S28/S17,0)</f>
+        <v/>
+      </c>
+      <c r="T30" s="26">
+        <f>IFERROR(T28/T17,0)</f>
+        <v/>
+      </c>
+      <c r="U30" s="26">
+        <f>IFERROR(U28/U17,0)</f>
+        <v/>
+      </c>
+      <c r="V30" s="26">
+        <f>IFERROR(V28/V17,0)</f>
+        <v/>
+      </c>
+      <c r="W30" s="26">
+        <f>IFERROR(W28/W17,0)</f>
+        <v/>
+      </c>
+      <c r="X30" s="26">
+        <f>IFERROR(X28/X17,0)</f>
+        <v/>
+      </c>
+      <c r="Y30" s="26">
+        <f>IFERROR(Y28/Y17,0)</f>
+        <v/>
+      </c>
+      <c r="Z30" s="16">
+        <f>IFERROR(Z28/Z17,0)</f>
         <v/>
       </c>
     </row>
@@ -4415,7 +4590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4471,7 +4646,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>-(Costs!$B$44+Costs!$B$45)</f>
+        <f>-(Costs!$B$50+Costs!$B$51)</f>
         <v/>
       </c>
     </row>
@@ -4482,7 +4657,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>-Tiers!$B$25*Costs!$B$46</f>
+        <f>-Tiers!$B$25*Costs!$B$52</f>
         <v/>
       </c>
     </row>
@@ -4510,7 +4685,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>-Costs!$B$23</f>
+        <f>-Costs!$B$29</f>
         <v/>
       </c>
     </row>
@@ -4521,168 +4696,179 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>MAX(0,Costs!$B$23-Tiers!$B$23)</f>
+        <f>MAX(0,Costs!$B$29-Tiers!$B$23)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Add-on margin per listing</t>
+        </is>
+      </c>
+      <c r="B11" s="27">
+        <f>IF(Tiers!$B$3="D. In-house media",Costs!$B$27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Contribution — listing-side transaction</t>
         </is>
       </c>
-      <c r="B11" s="21">
-        <f>B7+B9+B10</f>
-        <v/>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="B12" s="21">
+        <f>B7+B9+B10+B11</f>
+        <v/>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Negative here means every listing is a loss. That is the test.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Blended contribution per transaction</t>
         </is>
       </c>
-      <c r="B13" s="21">
-        <f>B7*(1-Scenarios!$E$11)+B11*Scenarios!$E$11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="B14" s="21">
+        <f>B7*(1-Scenarios!$E$11)+B12*Scenarios!$E$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Per agent, per month</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Membership fee</t>
-        </is>
-      </c>
-      <c r="B16" s="27">
-        <f>Tiers!$B$21</f>
-        <v/>
-      </c>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="20" t="n"/>
+      <c r="F16" s="20" t="n"/>
+      <c r="G16" s="20" t="n"/>
+      <c r="H16" s="20" t="n"/>
+      <c r="I16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Seat cost</t>
+          <t>Membership fee</t>
         </is>
       </c>
       <c r="B17" s="27">
-        <f>-(Costs!$B$41+Tiers!$B$24*Costs!$B$40)</f>
+        <f>Tiers!$B$21</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
+          <t>Seat cost</t>
+        </is>
+      </c>
+      <c r="B18" s="27">
+        <f>-(Costs!$B$47+Tiers!$B$24*Costs!$B$46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
           <t>Contribution from transactions</t>
         </is>
       </c>
-      <c r="B18" s="27">
-        <f>Scenarios!$E$10*B13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Contribution per agent per month</t>
-        </is>
-      </c>
-      <c r="B19" s="21">
-        <f>SUM(B16:B18)</f>
+      <c r="B19" s="27">
+        <f>Scenarios!$E$10*B14</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>Contribution per agent per month</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>SUM(B17:B19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>Contribution per agent per year</t>
         </is>
       </c>
-      <c r="B20" s="21">
-        <f>B19*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="B21" s="21">
+        <f>B20*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Break-even</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="n"/>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="20" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Fixed overhead per month</t>
-        </is>
-      </c>
-      <c r="B23" s="28">
-        <f>Costs!$B$37</f>
-        <v/>
-      </c>
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="20" t="n"/>
+      <c r="D23" s="20" t="n"/>
+      <c r="E23" s="20" t="n"/>
+      <c r="F23" s="20" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="20" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
+          <t>Fixed overhead per month</t>
+        </is>
+      </c>
+      <c r="B24" s="28">
+        <f>Costs!$B$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
           <t>Managing agent cost per month (year 1 average)</t>
         </is>
       </c>
-      <c r="B24" s="28">
+      <c r="B25" s="28">
         <f>AVERAGE('Managing Agent'!B30:M30)</f>
         <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Agents required to break even</t>
-        </is>
-      </c>
-      <c r="B25" s="14">
-        <f>IF(B19&lt;=0,"never",(B23+B24)/B19)</f>
-        <v/>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>If this says never, the architecture loses money on every agent and no amount of recruiting fixes it.</t>
-        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Agents required to break even</t>
+        </is>
+      </c>
+      <c r="B26" s="14">
+        <f>IF(B20&lt;=0,"never",(B24+B25)/B20)</f>
+        <v/>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>If this says never, the architecture loses money on every agent and no amount of recruiting fixes it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>Transactions per month required to break even</t>
         </is>
       </c>
-      <c r="B26" s="14">
-        <f>IF(B13&lt;=0,"never",(B23+B24)/B13)</f>
+      <c r="B27" s="14">
+        <f>IF(B14&lt;=0,"never",(B24+B25)/B14)</f>
         <v/>
       </c>
     </row>
@@ -6017,7 +6203,7 @@
         </is>
       </c>
       <c r="B16" s="28">
-        <f>SUM('P&amp;L'!N27:Y27)</f>
+        <f>SUM('P&amp;L'!N28:Y28)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Lean tech stack: drop DocuSign seats, CRM, and phone system
Form Simplicity Professional is free with Florida Realtors membership and does
transaction management; Ultimate adds unlimited e-signature for about $72-84 a
year, bought by the agent. So the brokerage needs one DocuSign seat for the
agent-packet PowerForm and nothing else per agent.

Per-agent cost drops from $83/month to $8 (email alias and storage). Fixed
overhead drops from $1,095 to $975. Break-even falls to roughly 6 agents across
every sensible fee structure, which makes the monthly fee a positioning choice
rather than a survival one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -2056,18 +2056,18 @@
         </is>
       </c>
       <c r="B36" s="17" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Base tier for a small firm.</t>
+          <t>Form Simplicity Professional is free with Florida Realtors membership and does transaction management. Upgrade only when volume demands it.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>E-signature</t>
+          <t>E-signature — broker seat only</t>
         </is>
       </c>
       <c r="B37" s="17" t="n">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>DocuSign Business Pro is about $45/user/month annually — needed for PowerForms.</t>
+          <t>DocuSign Business Pro, the one seat you need for the agent-packet PowerForm. Agents e-sign through Form Simplicity Ultimate, about $72-84/yr, which they buy.</t>
         </is>
       </c>
     </row>
@@ -2116,9 +2116,13 @@
         </is>
       </c>
       <c r="B40" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C40" s="12" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Agents use their own mobile. A brokerage phone system is overhead that buys you nothing.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -2175,30 +2179,30 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>CRM seat</t>
+          <t>CRM seat, if the brokerage provides one</t>
         </is>
       </c>
       <c r="B46" s="17" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Follow Up Boss class tool. Only charged for tiers that include it.</t>
+          <t>Lean stack: agents bring their own CRM or go without. Set to 65 if you decide to provide one.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>Email, storage, phone line</t>
+          <t>Email alias, storage, admin</t>
         </is>
       </c>
       <c r="B47" s="17" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Charged for every agent.</t>
+          <t>Google Workspace per seat. The only unavoidable per-agent cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set model defaults to the chosen structure: $29/month + $399/transaction
Architecture D with in-house media is now the default. At the lean stack this
breaks even at 7.3 agents or 4.3 closings a month, turns monthly profitable
around month 6, and recovers the cumulative deficit by month 11. Peak cash
requirement is about $1,700.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>B. Tiered</t>
+          <t>D. In-house media</t>
         </is>
       </c>
     </row>
@@ -1479,11 +1479,11 @@
         </is>
       </c>
       <c r="B17" s="17" t="n">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>The per-seat tech stack costs about $83 a month. A $20 fee cannot cover it; this one can.</t>
+          <t>Chosen structure. Works because the lean stack costs $8 per agent, not $83.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise cost stack to actual: E&O $80, no GL, dues prepaid, books in-house
Fixed monthly drops from $968 to $350. Break-even falls to 1.8 agents on cash
and 2.5 with the broker's time costed, which the brokerage already clears with
two licensees. Year-1 cash profit about $13.9k on the modest ramp.

Flags kept in the model rather than dropped silently: escrow still requires a
signed monthly reconciliation under Rule 61J2-14.012 whoever keeps the books,
E&O does not cover bodily injury at an open house, and association dues return
as a real cost in 2028.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -2004,11 +2004,11 @@
         </is>
       </c>
       <c r="B32" s="17" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Firm policy. Agents carry their own on top.</t>
+          <t>Your quoted premium.</t>
         </is>
       </c>
     </row>
@@ -2019,9 +2019,13 @@
         </is>
       </c>
       <c r="B33" s="17" t="n">
-        <v>45</v>
-      </c>
-      <c r="C33" s="12" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Declined. E&amp;O does not cover bodily injury at an open house — revisit before you host one.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -2030,11 +2034,11 @@
         </is>
       </c>
       <c r="B34" s="17" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Your own dues, annualized to a month.</t>
+          <t>Prepaid through 2027. The true annual cost is roughly $85/month; it returns in 2028.</t>
         </is>
       </c>
     </row>
@@ -2045,9 +2049,13 @@
         </is>
       </c>
       <c r="B35" s="17" t="n">
-        <v>35</v>
-      </c>
-      <c r="C35" s="12" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Vercel free tier and an Outlook account already paid for the year.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
@@ -2086,11 +2094,11 @@
         </is>
       </c>
       <c r="B38" s="17" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>Trust accounting is not a DIY job once agents are closing.</t>
+          <t>You are doing the books. Escrow still needs a signed monthly reconciliation under Rule 61J2-14.012 — see the Read Me.</t>
         </is>
       </c>
     </row>
@@ -2101,11 +2109,11 @@
         </is>
       </c>
       <c r="B39" s="17" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Annual attorney review amortized.</t>
+          <t>No retainer. Budget a one-time $800-1,500 for attorney review of the ICA and packet instead.</t>
         </is>
       </c>
     </row>
@@ -2131,9 +2139,13 @@
         </is>
       </c>
       <c r="B41" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="C41" s="12" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Often $0 with the right business account. Zero it once you confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
@@ -2198,11 +2210,11 @@
         </is>
       </c>
       <c r="B47" s="17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Google Workspace per seat. The only unavoidable per-agent cost.</t>
+          <t>Microsoft 365 aliases forwarding to the agent's own inbox cost nothing. A real mailbox per agent is about $6.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix broken cross-sheet references: rename the P&L tab
Excel cannot parse an unquoted sheet name containing "&". "=P&L!B8" was being
reinterpreted as an external workbook link, which is why opening the file in
SharePoint produced
=@P&'https://.../Documents/[L]L'!B8*$B$6

Renamed the tab to "Profit and Loss" and quoted every reference to it. Verified
no unquoted reference containing a space or ampersand remains anywhere in the
workbook.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance/TrueNorth-Pro-Forma.xlsx
+++ b/finance/TrueNorth-Pro-Forma.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Costs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="P&amp;L" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Profit and Loss" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Unit Economics" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Managing Agent" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="PM and EV" sheetId="7" state="visible" r:id="rId7"/>
@@ -1582,7 +1582,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P&amp;L — 24 months</t>
+          <t>Profit and Loss — 24 months</t>
         </is>
       </c>
     </row>
@@ -4451,99 +4451,99 @@
         </is>
       </c>
       <c r="B21" s="25">
-        <f>P&amp;L!B8*$B$6</f>
+        <f>'Profit and Loss'!B8*$B$6</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>P&amp;L!C8*$B$6</f>
+        <f>'Profit and Loss'!C8*$B$6</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>P&amp;L!D8*$B$6</f>
+        <f>'Profit and Loss'!D8*$B$6</f>
         <v/>
       </c>
       <c r="E21" s="25">
-        <f>P&amp;L!E8*$B$6</f>
+        <f>'Profit and Loss'!E8*$B$6</f>
         <v/>
       </c>
       <c r="F21" s="25">
-        <f>P&amp;L!F8*$B$6</f>
+        <f>'Profit and Loss'!F8*$B$6</f>
         <v/>
       </c>
       <c r="G21" s="25">
-        <f>P&amp;L!G8*$B$6</f>
+        <f>'Profit and Loss'!G8*$B$6</f>
         <v/>
       </c>
       <c r="H21" s="25">
-        <f>P&amp;L!H8*$B$6</f>
+        <f>'Profit and Loss'!H8*$B$6</f>
         <v/>
       </c>
       <c r="I21" s="25">
-        <f>P&amp;L!I8*$B$6</f>
+        <f>'Profit and Loss'!I8*$B$6</f>
         <v/>
       </c>
       <c r="J21" s="25">
-        <f>P&amp;L!J8*$B$6</f>
+        <f>'Profit and Loss'!J8*$B$6</f>
         <v/>
       </c>
       <c r="K21" s="25">
-        <f>P&amp;L!K8*$B$6</f>
+        <f>'Profit and Loss'!K8*$B$6</f>
         <v/>
       </c>
       <c r="L21" s="25">
-        <f>P&amp;L!L8*$B$6</f>
+        <f>'Profit and Loss'!L8*$B$6</f>
         <v/>
       </c>
       <c r="M21" s="25">
-        <f>P&amp;L!M8*$B$6</f>
+        <f>'Profit and Loss'!M8*$B$6</f>
         <v/>
       </c>
       <c r="N21" s="25">
-        <f>P&amp;L!N8*$B$6</f>
+        <f>'Profit and Loss'!N8*$B$6</f>
         <v/>
       </c>
       <c r="O21" s="25">
-        <f>P&amp;L!O8*$B$6</f>
+        <f>'Profit and Loss'!O8*$B$6</f>
         <v/>
       </c>
       <c r="P21" s="25">
-        <f>P&amp;L!P8*$B$6</f>
+        <f>'Profit and Loss'!P8*$B$6</f>
         <v/>
       </c>
       <c r="Q21" s="25">
-        <f>P&amp;L!Q8*$B$6</f>
+        <f>'Profit and Loss'!Q8*$B$6</f>
         <v/>
       </c>
       <c r="R21" s="25">
-        <f>P&amp;L!R8*$B$6</f>
+        <f>'Profit and Loss'!R8*$B$6</f>
         <v/>
       </c>
       <c r="S21" s="25">
-        <f>P&amp;L!S8*$B$6</f>
+        <f>'Profit and Loss'!S8*$B$6</f>
         <v/>
       </c>
       <c r="T21" s="25">
-        <f>P&amp;L!T8*$B$6</f>
+        <f>'Profit and Loss'!T8*$B$6</f>
         <v/>
       </c>
       <c r="U21" s="25">
-        <f>P&amp;L!U8*$B$6</f>
+        <f>'Profit and Loss'!U8*$B$6</f>
         <v/>
       </c>
       <c r="V21" s="25">
-        <f>P&amp;L!V8*$B$6</f>
+        <f>'Profit and Loss'!V8*$B$6</f>
         <v/>
       </c>
       <c r="W21" s="25">
-        <f>P&amp;L!W8*$B$6</f>
+        <f>'Profit and Loss'!W8*$B$6</f>
         <v/>
       </c>
       <c r="X21" s="25">
-        <f>P&amp;L!X8*$B$6</f>
+        <f>'Profit and Loss'!X8*$B$6</f>
         <v/>
       </c>
       <c r="Y21" s="25">
-        <f>P&amp;L!Y8*$B$6</f>
+        <f>'Profit and Loss'!Y8*$B$6</f>
         <v/>
       </c>
       <c r="Z21" s="13">
@@ -4669,95 +4669,95 @@
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>MAX(0,P&amp;L!C7-P&amp;L!B7)</f>
+        <f>MAX(0,'Profit and Loss'!C7-'Profit and Loss'!B7)</f>
         <v/>
       </c>
       <c r="D23" s="25">
-        <f>MAX(0,P&amp;L!D7-P&amp;L!C7)</f>
+        <f>MAX(0,'Profit and Loss'!D7-'Profit and Loss'!C7)</f>
         <v/>
       </c>
       <c r="E23" s="25">
-        <f>MAX(0,P&amp;L!E7-P&amp;L!D7)</f>
+        <f>MAX(0,'Profit and Loss'!E7-'Profit and Loss'!D7)</f>
         <v/>
       </c>
       <c r="F23" s="25">
-        <f>MAX(0,P&amp;L!F7-P&amp;L!E7)</f>
+        <f>MAX(0,'Profit and Loss'!F7-'Profit and Loss'!E7)</f>
         <v/>
       </c>
       <c r="G23" s="25">
-        <f>MAX(0,P&amp;L!G7-P&amp;L!F7)</f>
+        <f>MAX(0,'Profit and Loss'!G7-'Profit and Loss'!F7)</f>
         <v/>
       </c>
       <c r="H23" s="25">
-        <f>MAX(0,P&amp;L!H7-P&amp;L!G7)</f>
+        <f>MAX(0,'Profit and Loss'!H7-'Profit and Loss'!G7)</f>
         <v/>
       </c>
       <c r="I23" s="25">
-        <f>MAX(0,P&amp;L!I7-P&amp;L!H7)</f>
+        <f>MAX(0,'Profit and Loss'!I7-'Profit and Loss'!H7)</f>
         <v/>
       </c>
       <c r="J23" s="25">
-        <f>MAX(0,P&amp;L!J7-P&amp;L!I7)</f>
+        <f>MAX(0,'Profit and Loss'!J7-'Profit and Loss'!I7)</f>
         <v/>
       </c>
       <c r="K23" s="25">
-        <f>MAX(0,P&amp;L!K7-P&amp;L!J7)</f>
+        <f>MAX(0,'Profit and Loss'!K7-'Profit and Loss'!J7)</f>
         <v/>
       </c>
       <c r="L23" s="25">
-        <f>MAX(0,P&amp;L!L7-P&amp;L!K7)</f>
+        <f>MAX(0,'Profit and Loss'!L7-'Profit and Loss'!K7)</f>
         <v/>
       </c>
       <c r="M23" s="25">
-        <f>MAX(0,P&amp;L!M7-P&amp;L!L7)</f>
+        <f>MAX(0,'Profit and Loss'!M7-'Profit and Loss'!L7)</f>
         <v/>
       </c>
       <c r="N23" s="25">
-        <f>MAX(0,P&amp;L!N7-P&amp;L!M7)</f>
+        <f>MAX(0,'Profit and Loss'!N7-'Profit and Loss'!M7)</f>
         <v/>
       </c>
       <c r="O23" s="25">
-        <f>MAX(0,P&amp;L!O7-P&amp;L!N7)</f>
+        <f>MAX(0,'Profit and Loss'!O7-'Profit and Loss'!N7)</f>
         <v/>
       </c>
       <c r="P23" s="25">
-        <f>MAX(0,P&amp;L!P7-P&amp;L!O7)</f>
+        <f>MAX(0,'Profit and Loss'!P7-'Profit and Loss'!O7)</f>
         <v/>
       </c>
       <c r="Q23" s="25">
-        <f>MAX(0,P&amp;L!Q7-P&amp;L!P7)</f>
+        <f>MAX(0,'Profit and Loss'!Q7-'Profit and Loss'!P7)</f>
         <v/>
       </c>
       <c r="R23" s="25">
-        <f>MAX(0,P&amp;L!R7-P&amp;L!Q7)</f>
+        <f>MAX(0,'Profit and Loss'!R7-'Profit and Loss'!Q7)</f>
         <v/>
       </c>
       <c r="S23" s="25">
-        <f>MAX(0,P&amp;L!S7-P&amp;L!R7)</f>
+        <f>MAX(0,'Profit and Loss'!S7-'Profit and Loss'!R7)</f>
         <v/>
       </c>
       <c r="T23" s="25">
-        <f>MAX(0,P&amp;L!T7-P&amp;L!S7)</f>
+        <f>MAX(0,'Profit and Loss'!T7-'Profit and Loss'!S7)</f>
         <v/>
       </c>
       <c r="U23" s="25">
-        <f>MAX(0,P&amp;L!U7-P&amp;L!T7)</f>
+        <f>MAX(0,'Profit and Loss'!U7-'Profit and Loss'!T7)</f>
         <v/>
       </c>
       <c r="V23" s="25">
-        <f>MAX(0,P&amp;L!V7-P&amp;L!U7)</f>
+        <f>MAX(0,'Profit and Loss'!V7-'Profit and Loss'!U7)</f>
         <v/>
       </c>
       <c r="W23" s="25">
-        <f>MAX(0,P&amp;L!W7-P&amp;L!V7)</f>
+        <f>MAX(0,'Profit and Loss'!W7-'Profit and Loss'!V7)</f>
         <v/>
       </c>
       <c r="X23" s="25">
-        <f>MAX(0,P&amp;L!X7-P&amp;L!W7)</f>
+        <f>MAX(0,'Profit and Loss'!X7-'Profit and Loss'!W7)</f>
         <v/>
       </c>
       <c r="Y23" s="25">
-        <f>MAX(0,P&amp;L!Y7-P&amp;L!X7)</f>
+        <f>MAX(0,'Profit and Loss'!Y7-'Profit and Loss'!X7)</f>
         <v/>
       </c>
       <c r="Z23" s="13">
@@ -5324,7 +5324,7 @@
         </is>
       </c>
       <c r="B14" s="28">
-        <f>SUM('P&amp;L'!N28:Y28)</f>
+        <f>SUM('Profit and Loss'!N28:Y28)</f>
         <v/>
       </c>
     </row>

</xml_diff>